<commit_message>
Point the Vercel import at the new courses repo; refresh the URL workbook
The CHART courses moved from estesstite to me5231979/courses, so the import
list targets that repo instead. The workbook now carries explicit path
columns per edition (correct for the move), a Paths by Repo tab for the two
repos that hold many courses, and URLs built by concatenating the domain
with the path.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CHUxqeQb2UgQw5JmmaoKqy
</commit_message>
<xml_diff>
--- a/docs/Vanderbilt-Learning-Series-URLs.xlsx
+++ b/docs/Vanderbilt-Learning-Series-URLs.xlsx
@@ -9,10 +9,11 @@
   <sheets>
     <sheet name="Repos to Import" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Course URLs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Setup Checklist" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Paths by Repo" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Setup Checklist" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Course URLs'!$A$3:$L$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Course URLs'!$A$3:$N$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -91,6 +92,10 @@
       <sz val="10"/>
     </font>
     <font>
+      <name val="Courier New"/>
+      <sz val="10"/>
+    </font>
+    <font>
       <name val="Arial"/>
       <color rgb="001E7B34"/>
       <sz val="10"/>
@@ -150,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -219,6 +224,9 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -231,16 +239,23 @@
     <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -614,8 +629,8 @@
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -625,10 +640,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Import each repo as ONE Vercel project. Root Directory stays EMPTY and there is no build command: all three editions are pre-generated static files served from one deployment. Fill the yellow column as each import finishes and the Course URLs tab updates itself.</t>
+          <t>One repo becomes one Vercel project. Root Directory stays EMPTY and there is no build command. Paste each project's domain into the yellow column and every URL on the other tabs fills itself in.</t>
         </is>
       </c>
     </row>
@@ -660,7 +675,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Courses served</t>
+          <t>Courses</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -849,7 +864,7 @@
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
-          <t>Repo is TeamUp; the course is called Building Brave Teams.</t>
+          <t>Repo is TeamUp; the course is Building Brave Teams.</t>
         </is>
       </c>
     </row>
@@ -912,17 +927,17 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>estesstite</t>
+          <t>courses</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>https://github.com/me5231979/estesstite</t>
+          <t>https://github.com/me5231979/courses</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>chart-program</t>
+          <t>chart-courses</t>
         </is>
       </c>
       <c r="D12" s="15" t="inlineStr">
@@ -937,7 +952,7 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>Hosts 7 courses under /learn/. Biggest single import after the library.</t>
+          <t>NEW. The 7 CHART courses, moved out of estesstite. Import this instead of estesstite.</t>
         </is>
       </c>
     </row>
@@ -969,7 +984,7 @@
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
-          <t>The catalog itself PLUS 13 courses hosted inside it. Import this one.</t>
+          <t>The catalog PLUS 13 courses inside it. Must be imported.</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1016,7 @@
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>AI 201. Live, but no longer carded on the library page.</t>
+          <t>AI 201. Live, no longer carded on the library page.</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1036,7 @@
       </c>
       <c r="G15" s="20" t="inlineStr">
         <is>
-          <t>Courses currently carded on the library page.</t>
+          <t>Courses carded on the library page.</t>
         </is>
       </c>
     </row>
@@ -1042,14 +1057,14 @@
     <row r="19">
       <c r="A19" s="23" t="inlineStr">
         <is>
-          <t>Example format: ai-classroom-one.vercel.app  (no https://, no trailing slash)</t>
+          <t>Format: ai-classroom-one.vercel.app   (no https://, no trailing slash)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="23" t="inlineStr">
         <is>
-          <t>Vercel assigns a random suffix because plain names are taken globally. A custom domain is the fix.</t>
+          <t>estesstite is deliberately absent: its 7 courses now live in the courses repo.</t>
         </is>
       </c>
     </row>
@@ -1080,21 +1095,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="52" customWidth="1" min="7" max="7"/>
-    <col width="54" customWidth="1" min="8" max="8"/>
-    <col width="52" customWidth="1" min="9" max="9"/>
-    <col width="52" customWidth="1" min="10" max="10"/>
-    <col width="52" customWidth="1" min="11" max="11"/>
-    <col width="54" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
+    <col width="48" customWidth="1" min="11" max="11"/>
+    <col width="48" customWidth="1" min="12" max="12"/>
+    <col width="48" customWidth="1" min="13" max="13"/>
+    <col width="50" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1104,10 +1121,10 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Columns F to I are live today on GitHub Pages. Columns J to L build themselves from the Vercel domain you enter on the Repos tab, and stay blank until you do.</t>
+          <t>Columns F to H are the paths that go after the domain. I to K build the live Vercel links from the domain on the Repos tab. L to N are today's GitHub Pages links, kept for reference until the switch.</t>
         </is>
       </c>
     </row>
@@ -1139,37 +1156,47 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Classroom (live)</t>
+          <t>Classroom path</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Self-paced (live)</t>
+          <t>Self-paced path</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Facilitator (live)</t>
+          <t>Facilitator path</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Syllabus (live)</t>
+          <t>Classroom URL</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Classroom (Vercel)</t>
+          <t>Self-paced URL</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Self-paced (Vercel)</t>
+          <t>Facilitator URL</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>Facilitator (Vercel)</t>
+          <t>Classroom (live today)</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Self-paced (live today)</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>Facilitator (live today)</t>
         </is>
       </c>
     </row>
@@ -1199,46 +1226,56 @@
           <t>Coaching-for-Performance</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="27" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G4" s="27" t="inlineStr">
+        <is>
+          <t>/web/</t>
+        </is>
+      </c>
+      <c r="H4" s="27" t="inlineStr">
+        <is>
+          <t>/facilitator/</t>
+        </is>
+      </c>
+      <c r="I4" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E4,'Repos to Import'!$A$4:$A$14,0))="",F4=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E4,'Repos to Import'!$A$4:$A$14,0))&amp;F4),"")</f>
+        <v/>
+      </c>
+      <c r="J4" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E4,'Repos to Import'!$A$4:$A$14,0))="",G4=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E4,'Repos to Import'!$A$4:$A$14,0))&amp;G4),"")</f>
+        <v/>
+      </c>
+      <c r="K4" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E4,'Repos to Import'!$A$4:$A$14,0))="",H4=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E4,'Repos to Import'!$A$4:$A$14,0))&amp;H4),"")</f>
+        <v/>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Coaching-for-Performance/</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Coaching-for-Performance/web/</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Coaching-for-Performance/facilitator/</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-coaching-for-performance.html</t>
-        </is>
-      </c>
-      <c r="J4" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E4,'Repos to Import'!$A$4:$A$14,0))="",F4=""),"",SUBSTITUTE(F4,"https://me5231979.github.io/"&amp;$E4&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E4,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K4" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E4,'Repos to Import'!$A$4:$A$14,0))="",G4=""),"",SUBSTITUTE(G4,"https://me5231979.github.io/"&amp;$E4&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E4,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L4" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E4,'Repos to Import'!$A$4:$A$14,0))="",H4=""),"",SUBSTITUTE(H4,"https://me5231979.github.io/"&amp;$E4&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E4,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>Change That Sticks</t>
         </is>
       </c>
-      <c r="B5" s="29" t="inlineStr">
+      <c r="B5" s="30" t="inlineStr">
         <is>
           <t>Manager Voyage</t>
         </is>
@@ -1248,7 +1285,7 @@
           <t>ai leadership</t>
         </is>
       </c>
-      <c r="D5" s="30" t="inlineStr">
+      <c r="D5" s="31" t="inlineStr">
         <is>
           <t>Classroom 90 min · Self-paced ~45 min</t>
         </is>
@@ -1258,37 +1295,47 @@
           <t>Course_Library</t>
         </is>
       </c>
-      <c r="F5" s="11" t="inlineStr">
+      <c r="F5" s="32" t="inlineStr">
+        <is>
+          <t>/courses/Change-Leadership-for-AI/</t>
+        </is>
+      </c>
+      <c r="G5" s="32" t="inlineStr">
+        <is>
+          <t>/courses/Change-Leadership-for-AI/web/</t>
+        </is>
+      </c>
+      <c r="H5" s="32" t="inlineStr">
+        <is>
+          <t>/courses/Change-Leadership-for-AI/facilitator/</t>
+        </is>
+      </c>
+      <c r="I5" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E5,'Repos to Import'!$A$4:$A$14,0))="",F5=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E5,'Repos to Import'!$A$4:$A$14,0))&amp;F5),"")</f>
+        <v/>
+      </c>
+      <c r="J5" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E5,'Repos to Import'!$A$4:$A$14,0))="",G5=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E5,'Repos to Import'!$A$4:$A$14,0))&amp;G5),"")</f>
+        <v/>
+      </c>
+      <c r="K5" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E5,'Repos to Import'!$A$4:$A$14,0))="",H5=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E5,'Repos to Import'!$A$4:$A$14,0))&amp;H5),"")</f>
+        <v/>
+      </c>
+      <c r="L5" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Change-Leadership-for-AI/</t>
         </is>
       </c>
-      <c r="G5" s="11" t="inlineStr">
+      <c r="M5" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Change-Leadership-for-AI/web/</t>
         </is>
       </c>
-      <c r="H5" s="11" t="inlineStr">
+      <c r="N5" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Change-Leadership-for-AI/facilitator/</t>
         </is>
-      </c>
-      <c r="I5" s="11" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-change-leadership-for-ai.html</t>
-        </is>
-      </c>
-      <c r="J5" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E5,'Repos to Import'!$A$4:$A$14,0))="",F5=""),"",SUBSTITUTE(F5,"https://me5231979.github.io/"&amp;$E5&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E5,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K5" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E5,'Repos to Import'!$A$4:$A$14,0))="",G5=""),"",SUBSTITUTE(G5,"https://me5231979.github.io/"&amp;$E5&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E5,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L5" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E5,'Repos to Import'!$A$4:$A$14,0))="",H5=""),"",SUBSTITUTE(H5,"https://me5231979.github.io/"&amp;$E5&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E5,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
       </c>
     </row>
     <row r="6">
@@ -1317,46 +1364,56 @@
           <t>Course_Library</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="27" t="inlineStr">
+        <is>
+          <t>/courses/Delegating-with-AI/</t>
+        </is>
+      </c>
+      <c r="G6" s="27" t="inlineStr">
+        <is>
+          <t>/courses/Delegating-with-AI/web/</t>
+        </is>
+      </c>
+      <c r="H6" s="27" t="inlineStr">
+        <is>
+          <t>/courses/Delegating-with-AI/facilitator/</t>
+        </is>
+      </c>
+      <c r="I6" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E6,'Repos to Import'!$A$4:$A$14,0))="",F6=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E6,'Repos to Import'!$A$4:$A$14,0))&amp;F6),"")</f>
+        <v/>
+      </c>
+      <c r="J6" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E6,'Repos to Import'!$A$4:$A$14,0))="",G6=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E6,'Repos to Import'!$A$4:$A$14,0))&amp;G6),"")</f>
+        <v/>
+      </c>
+      <c r="K6" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E6,'Repos to Import'!$A$4:$A$14,0))="",H6=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E6,'Repos to Import'!$A$4:$A$14,0))&amp;H6),"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Delegating-with-AI/</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="M6" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Delegating-with-AI/web/</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="N6" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Delegating-with-AI/facilitator/</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-delegating-with-ai.html</t>
-        </is>
-      </c>
-      <c r="J6" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E6,'Repos to Import'!$A$4:$A$14,0))="",F6=""),"",SUBSTITUTE(F6,"https://me5231979.github.io/"&amp;$E6&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E6,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K6" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E6,'Repos to Import'!$A$4:$A$14,0))="",G6=""),"",SUBSTITUTE(G6,"https://me5231979.github.io/"&amp;$E6&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E6,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L6" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E6,'Repos to Import'!$A$4:$A$14,0))="",H6=""),"",SUBSTITUTE(H6,"https://me5231979.github.io/"&amp;$E6&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E6,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="inlineStr">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>Feedback, Ready</t>
         </is>
       </c>
-      <c r="B7" s="29" t="inlineStr">
+      <c r="B7" s="30" t="inlineStr">
         <is>
           <t>Manager Voyage</t>
         </is>
@@ -1366,7 +1423,7 @@
           <t>ai leadership</t>
         </is>
       </c>
-      <c r="D7" s="30" t="inlineStr">
+      <c r="D7" s="31" t="inlineStr">
         <is>
           <t>Classroom 40 min · Self-paced ~15 min</t>
         </is>
@@ -1376,37 +1433,47 @@
           <t>Course_Library</t>
         </is>
       </c>
-      <c r="F7" s="11" t="inlineStr">
+      <c r="F7" s="32" t="inlineStr">
+        <is>
+          <t>/ai-coaching-feedback/</t>
+        </is>
+      </c>
+      <c r="G7" s="32" t="inlineStr">
+        <is>
+          <t>/ai-coaching-feedback/web/</t>
+        </is>
+      </c>
+      <c r="H7" s="32" t="inlineStr">
+        <is>
+          <t>/ai-coaching-feedback/facilitator/</t>
+        </is>
+      </c>
+      <c r="I7" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E7,'Repos to Import'!$A$4:$A$14,0))="",F7=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E7,'Repos to Import'!$A$4:$A$14,0))&amp;F7),"")</f>
+        <v/>
+      </c>
+      <c r="J7" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E7,'Repos to Import'!$A$4:$A$14,0))="",G7=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E7,'Repos to Import'!$A$4:$A$14,0))&amp;G7),"")</f>
+        <v/>
+      </c>
+      <c r="K7" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E7,'Repos to Import'!$A$4:$A$14,0))="",H7=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E7,'Repos to Import'!$A$4:$A$14,0))&amp;H7),"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/ai-coaching-feedback/</t>
         </is>
       </c>
-      <c r="G7" s="11" t="inlineStr">
+      <c r="M7" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/ai-coaching-feedback/web/</t>
         </is>
       </c>
-      <c r="H7" s="11" t="inlineStr">
+      <c r="N7" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/ai-coaching-feedback/facilitator/</t>
         </is>
-      </c>
-      <c r="I7" s="11" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-ai-coaching-feedback.html</t>
-        </is>
-      </c>
-      <c r="J7" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E7,'Repos to Import'!$A$4:$A$14,0))="",F7=""),"",SUBSTITUTE(F7,"https://me5231979.github.io/"&amp;$E7&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E7,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K7" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E7,'Repos to Import'!$A$4:$A$14,0))="",G7=""),"",SUBSTITUTE(G7,"https://me5231979.github.io/"&amp;$E7&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E7,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L7" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E7,'Repos to Import'!$A$4:$A$14,0))="",H7=""),"",SUBSTITUTE(H7,"https://me5231979.github.io/"&amp;$E7&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E7,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
       </c>
     </row>
     <row r="8">
@@ -1435,46 +1502,56 @@
           <t>Course_Library</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="27" t="inlineStr">
+        <is>
+          <t>/courses/Hiring-with-AI/</t>
+        </is>
+      </c>
+      <c r="G8" s="27" t="inlineStr">
+        <is>
+          <t>/courses/Hiring-with-AI/web/</t>
+        </is>
+      </c>
+      <c r="H8" s="27" t="inlineStr">
+        <is>
+          <t>/courses/Hiring-with-AI/facilitator/</t>
+        </is>
+      </c>
+      <c r="I8" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E8,'Repos to Import'!$A$4:$A$14,0))="",F8=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E8,'Repos to Import'!$A$4:$A$14,0))&amp;F8),"")</f>
+        <v/>
+      </c>
+      <c r="J8" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E8,'Repos to Import'!$A$4:$A$14,0))="",G8=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E8,'Repos to Import'!$A$4:$A$14,0))&amp;G8),"")</f>
+        <v/>
+      </c>
+      <c r="K8" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E8,'Repos to Import'!$A$4:$A$14,0))="",H8=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E8,'Repos to Import'!$A$4:$A$14,0))&amp;H8),"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Hiring-with-AI/</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="M8" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Hiring-with-AI/web/</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="N8" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Hiring-with-AI/facilitator/</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-hiring-with-ai.html</t>
-        </is>
-      </c>
-      <c r="J8" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E8,'Repos to Import'!$A$4:$A$14,0))="",F8=""),"",SUBSTITUTE(F8,"https://me5231979.github.io/"&amp;$E8&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E8,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K8" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E8,'Repos to Import'!$A$4:$A$14,0))="",G8=""),"",SUBSTITUTE(G8,"https://me5231979.github.io/"&amp;$E8&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E8,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L8" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E8,'Repos to Import'!$A$4:$A$14,0))="",H8=""),"",SUBSTITUTE(H8,"https://me5231979.github.io/"&amp;$E8&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E8,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
     </row>
     <row r="9">
-      <c r="A9" s="28" t="inlineStr">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>Leading the Shift</t>
         </is>
       </c>
-      <c r="B9" s="29" t="inlineStr">
+      <c r="B9" s="30" t="inlineStr">
         <is>
           <t>Manager Voyage</t>
         </is>
@@ -1484,7 +1561,7 @@
           <t>ai leadership</t>
         </is>
       </c>
-      <c r="D9" s="30" t="inlineStr">
+      <c r="D9" s="31" t="inlineStr">
         <is>
           <t>Classroom 40 min · Self-paced ~15 min</t>
         </is>
@@ -1494,37 +1571,47 @@
           <t>Course_Library</t>
         </is>
       </c>
-      <c r="F9" s="11" t="inlineStr">
+      <c r="F9" s="32" t="inlineStr">
+        <is>
+          <t>/leading-ai-adoption/</t>
+        </is>
+      </c>
+      <c r="G9" s="32" t="inlineStr">
+        <is>
+          <t>/leading-ai-adoption/web/</t>
+        </is>
+      </c>
+      <c r="H9" s="32" t="inlineStr">
+        <is>
+          <t>/leading-ai-adoption/facilitator/</t>
+        </is>
+      </c>
+      <c r="I9" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E9,'Repos to Import'!$A$4:$A$14,0))="",F9=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E9,'Repos to Import'!$A$4:$A$14,0))&amp;F9),"")</f>
+        <v/>
+      </c>
+      <c r="J9" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E9,'Repos to Import'!$A$4:$A$14,0))="",G9=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E9,'Repos to Import'!$A$4:$A$14,0))&amp;G9),"")</f>
+        <v/>
+      </c>
+      <c r="K9" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E9,'Repos to Import'!$A$4:$A$14,0))="",H9=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E9,'Repos to Import'!$A$4:$A$14,0))&amp;H9),"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/leading-ai-adoption/</t>
         </is>
       </c>
-      <c r="G9" s="11" t="inlineStr">
+      <c r="M9" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/leading-ai-adoption/web/</t>
         </is>
       </c>
-      <c r="H9" s="11" t="inlineStr">
+      <c r="N9" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/leading-ai-adoption/facilitator/</t>
         </is>
-      </c>
-      <c r="I9" s="11" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-leading-ai-adoption.html</t>
-        </is>
-      </c>
-      <c r="J9" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E9,'Repos to Import'!$A$4:$A$14,0))="",F9=""),"",SUBSTITUTE(F9,"https://me5231979.github.io/"&amp;$E9&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E9,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K9" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E9,'Repos to Import'!$A$4:$A$14,0))="",G9=""),"",SUBSTITUTE(G9,"https://me5231979.github.io/"&amp;$E9&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E9,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L9" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E9,'Repos to Import'!$A$4:$A$14,0))="",H9=""),"",SUBSTITUTE(H9,"https://me5231979.github.io/"&amp;$E9&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E9,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
       </c>
     </row>
     <row r="10">
@@ -1553,46 +1640,56 @@
           <t>Course_Library</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="27" t="inlineStr">
+        <is>
+          <t>/courses/Leading-AI-Adoption/</t>
+        </is>
+      </c>
+      <c r="G10" s="27" t="inlineStr">
+        <is>
+          <t>/courses/Leading-AI-Adoption/web/</t>
+        </is>
+      </c>
+      <c r="H10" s="27" t="inlineStr">
+        <is>
+          <t>/courses/Leading-AI-Adoption/facilitator/</t>
+        </is>
+      </c>
+      <c r="I10" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E10,'Repos to Import'!$A$4:$A$14,0))="",F10=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E10,'Repos to Import'!$A$4:$A$14,0))&amp;F10),"")</f>
+        <v/>
+      </c>
+      <c r="J10" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E10,'Repos to Import'!$A$4:$A$14,0))="",G10=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E10,'Repos to Import'!$A$4:$A$14,0))&amp;G10),"")</f>
+        <v/>
+      </c>
+      <c r="K10" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E10,'Repos to Import'!$A$4:$A$14,0))="",H10=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E10,'Repos to Import'!$A$4:$A$14,0))&amp;H10),"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Leading-AI-Adoption/</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="M10" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Leading-AI-Adoption/web/</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="N10" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Leading-AI-Adoption/facilitator/</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-making-ai-normal.html</t>
-        </is>
-      </c>
-      <c r="J10" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E10,'Repos to Import'!$A$4:$A$14,0))="",F10=""),"",SUBSTITUTE(F10,"https://me5231979.github.io/"&amp;$E10&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E10,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K10" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E10,'Repos to Import'!$A$4:$A$14,0))="",G10=""),"",SUBSTITUTE(G10,"https://me5231979.github.io/"&amp;$E10&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E10,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L10" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E10,'Repos to Import'!$A$4:$A$14,0))="",H10=""),"",SUBSTITUTE(H10,"https://me5231979.github.io/"&amp;$E10&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E10,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
     </row>
     <row r="11">
-      <c r="A11" s="28" t="inlineStr">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>People Data, Safely</t>
         </is>
       </c>
-      <c r="B11" s="29" t="inlineStr">
+      <c r="B11" s="30" t="inlineStr">
         <is>
           <t>Manager Voyage</t>
         </is>
@@ -1602,7 +1699,7 @@
           <t>ai leadership</t>
         </is>
       </c>
-      <c r="D11" s="30" t="inlineStr">
+      <c r="D11" s="31" t="inlineStr">
         <is>
           <t>Classroom 90 min · Self-paced ~45 min</t>
         </is>
@@ -1612,37 +1709,47 @@
           <t>Course_Library</t>
         </is>
       </c>
-      <c r="F11" s="11" t="inlineStr">
+      <c r="F11" s="32" t="inlineStr">
+        <is>
+          <t>/courses/People-Data-with-AI/</t>
+        </is>
+      </c>
+      <c r="G11" s="32" t="inlineStr">
+        <is>
+          <t>/courses/People-Data-with-AI/web/</t>
+        </is>
+      </c>
+      <c r="H11" s="32" t="inlineStr">
+        <is>
+          <t>/courses/People-Data-with-AI/facilitator/</t>
+        </is>
+      </c>
+      <c r="I11" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E11,'Repos to Import'!$A$4:$A$14,0))="",F11=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E11,'Repos to Import'!$A$4:$A$14,0))&amp;F11),"")</f>
+        <v/>
+      </c>
+      <c r="J11" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E11,'Repos to Import'!$A$4:$A$14,0))="",G11=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E11,'Repos to Import'!$A$4:$A$14,0))&amp;G11),"")</f>
+        <v/>
+      </c>
+      <c r="K11" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E11,'Repos to Import'!$A$4:$A$14,0))="",H11=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E11,'Repos to Import'!$A$4:$A$14,0))&amp;H11),"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/People-Data-with-AI/</t>
         </is>
       </c>
-      <c r="G11" s="11" t="inlineStr">
+      <c r="M11" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/People-Data-with-AI/web/</t>
         </is>
       </c>
-      <c r="H11" s="11" t="inlineStr">
+      <c r="N11" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/People-Data-with-AI/facilitator/</t>
         </is>
-      </c>
-      <c r="I11" s="11" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-people-data-with-ai.html</t>
-        </is>
-      </c>
-      <c r="J11" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E11,'Repos to Import'!$A$4:$A$14,0))="",F11=""),"",SUBSTITUTE(F11,"https://me5231979.github.io/"&amp;$E11&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E11,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K11" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E11,'Repos to Import'!$A$4:$A$14,0))="",G11=""),"",SUBSTITUTE(G11,"https://me5231979.github.io/"&amp;$E11&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E11,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L11" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E11,'Repos to Import'!$A$4:$A$14,0))="",H11=""),"",SUBSTITUTE(H11,"https://me5231979.github.io/"&amp;$E11&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E11,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
       </c>
     </row>
     <row r="12">
@@ -1671,46 +1778,56 @@
           <t>Course_Library</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F12" s="27" t="inlineStr">
+        <is>
+          <t>/ai-talent-decisions/</t>
+        </is>
+      </c>
+      <c r="G12" s="27" t="inlineStr">
+        <is>
+          <t>/ai-talent-decisions/web/</t>
+        </is>
+      </c>
+      <c r="H12" s="27" t="inlineStr">
+        <is>
+          <t>/ai-talent-decisions/facilitator/</t>
+        </is>
+      </c>
+      <c r="I12" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E12,'Repos to Import'!$A$4:$A$14,0))="",F12=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E12,'Repos to Import'!$A$4:$A$14,0))&amp;F12),"")</f>
+        <v/>
+      </c>
+      <c r="J12" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E12,'Repos to Import'!$A$4:$A$14,0))="",G12=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E12,'Repos to Import'!$A$4:$A$14,0))&amp;G12),"")</f>
+        <v/>
+      </c>
+      <c r="K12" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E12,'Repos to Import'!$A$4:$A$14,0))="",H12=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E12,'Repos to Import'!$A$4:$A$14,0))&amp;H12),"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/ai-talent-decisions/</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="M12" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/ai-talent-decisions/web/</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="N12" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/ai-talent-decisions/facilitator/</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-ai-talent-decisions.html</t>
-        </is>
-      </c>
-      <c r="J12" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E12,'Repos to Import'!$A$4:$A$14,0))="",F12=""),"",SUBSTITUTE(F12,"https://me5231979.github.io/"&amp;$E12&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E12,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K12" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E12,'Repos to Import'!$A$4:$A$14,0))="",G12=""),"",SUBSTITUTE(G12,"https://me5231979.github.io/"&amp;$E12&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E12,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L12" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E12,'Repos to Import'!$A$4:$A$14,0))="",H12=""),"",SUBSTITUTE(H12,"https://me5231979.github.io/"&amp;$E12&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E12,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
     </row>
     <row r="13">
-      <c r="A13" s="28" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>Navigating Difficult Conversations</t>
         </is>
       </c>
-      <c r="B13" s="29" t="inlineStr">
+      <c r="B13" s="30" t="inlineStr">
         <is>
           <t>Manager Voyage</t>
         </is>
@@ -1720,7 +1837,7 @@
           <t>communication leadership</t>
         </is>
       </c>
-      <c r="D13" s="30" t="inlineStr">
+      <c r="D13" s="31" t="inlineStr">
         <is>
           <t>Classroom 90 min · Self-paced ~45 min</t>
         </is>
@@ -1730,37 +1847,47 @@
           <t>Difficult_Conversations</t>
         </is>
       </c>
-      <c r="F13" s="11" t="inlineStr">
+      <c r="F13" s="32" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G13" s="32" t="inlineStr">
+        <is>
+          <t>/web/</t>
+        </is>
+      </c>
+      <c r="H13" s="32" t="inlineStr">
+        <is>
+          <t>/facilitator/</t>
+        </is>
+      </c>
+      <c r="I13" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E13,'Repos to Import'!$A$4:$A$14,0))="",F13=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E13,'Repos to Import'!$A$4:$A$14,0))&amp;F13),"")</f>
+        <v/>
+      </c>
+      <c r="J13" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E13,'Repos to Import'!$A$4:$A$14,0))="",G13=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E13,'Repos to Import'!$A$4:$A$14,0))&amp;G13),"")</f>
+        <v/>
+      </c>
+      <c r="K13" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E13,'Repos to Import'!$A$4:$A$14,0))="",H13=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E13,'Repos to Import'!$A$4:$A$14,0))&amp;H13),"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Difficult_Conversations/</t>
         </is>
       </c>
-      <c r="G13" s="11" t="inlineStr">
+      <c r="M13" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Difficult_Conversations/web/</t>
         </is>
       </c>
-      <c r="H13" s="11" t="inlineStr">
+      <c r="N13" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Difficult_Conversations/facilitator/</t>
         </is>
-      </c>
-      <c r="I13" s="11" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-difficult-conversations.html</t>
-        </is>
-      </c>
-      <c r="J13" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E13,'Repos to Import'!$A$4:$A$14,0))="",F13=""),"",SUBSTITUTE(F13,"https://me5231979.github.io/"&amp;$E13&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E13,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K13" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E13,'Repos to Import'!$A$4:$A$14,0))="",G13=""),"",SUBSTITUTE(G13,"https://me5231979.github.io/"&amp;$E13&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E13,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L13" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E13,'Repos to Import'!$A$4:$A$14,0))="",H13=""),"",SUBSTITUTE(H13,"https://me5231979.github.io/"&amp;$E13&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E13,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
       </c>
     </row>
     <row r="14">
@@ -1789,46 +1916,56 @@
           <t>Emotional-Intelligence</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F14" s="27" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G14" s="27" t="inlineStr">
+        <is>
+          <t>/web/</t>
+        </is>
+      </c>
+      <c r="H14" s="27" t="inlineStr">
+        <is>
+          <t>/facilitator/</t>
+        </is>
+      </c>
+      <c r="I14" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E14,'Repos to Import'!$A$4:$A$14,0))="",F14=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E14,'Repos to Import'!$A$4:$A$14,0))&amp;F14),"")</f>
+        <v/>
+      </c>
+      <c r="J14" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E14,'Repos to Import'!$A$4:$A$14,0))="",G14=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E14,'Repos to Import'!$A$4:$A$14,0))&amp;G14),"")</f>
+        <v/>
+      </c>
+      <c r="K14" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E14,'Repos to Import'!$A$4:$A$14,0))="",H14=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E14,'Repos to Import'!$A$4:$A$14,0))&amp;H14),"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Emotional-Intelligence/</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="M14" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Emotional-Intelligence/web/</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="N14" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Emotional-Intelligence/facilitator/</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-emotional-intelligence.html</t>
-        </is>
-      </c>
-      <c r="J14" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E14,'Repos to Import'!$A$4:$A$14,0))="",F14=""),"",SUBSTITUTE(F14,"https://me5231979.github.io/"&amp;$E14&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E14,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K14" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E14,'Repos to Import'!$A$4:$A$14,0))="",G14=""),"",SUBSTITUTE(G14,"https://me5231979.github.io/"&amp;$E14&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E14,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L14" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E14,'Repos to Import'!$A$4:$A$14,0))="",H14=""),"",SUBSTITUTE(H14,"https://me5231979.github.io/"&amp;$E14&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E14,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="inlineStr">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>Presentation &amp; Public Speaking</t>
         </is>
       </c>
-      <c r="B15" s="29" t="inlineStr">
+      <c r="B15" s="30" t="inlineStr">
         <is>
           <t>Manager Voyage</t>
         </is>
@@ -1838,7 +1975,7 @@
           <t>communication leadership</t>
         </is>
       </c>
-      <c r="D15" s="30" t="inlineStr">
+      <c r="D15" s="31" t="inlineStr">
         <is>
           <t>Classroom 90 min · Self-paced ~45 min</t>
         </is>
@@ -1848,37 +1985,47 @@
           <t>Presentation-Public-Speaking</t>
         </is>
       </c>
-      <c r="F15" s="11" t="inlineStr">
+      <c r="F15" s="32" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G15" s="32" t="inlineStr">
+        <is>
+          <t>/web/</t>
+        </is>
+      </c>
+      <c r="H15" s="32" t="inlineStr">
+        <is>
+          <t>/facilitator/</t>
+        </is>
+      </c>
+      <c r="I15" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E15,'Repos to Import'!$A$4:$A$14,0))="",F15=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E15,'Repos to Import'!$A$4:$A$14,0))&amp;F15),"")</f>
+        <v/>
+      </c>
+      <c r="J15" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E15,'Repos to Import'!$A$4:$A$14,0))="",G15=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E15,'Repos to Import'!$A$4:$A$14,0))&amp;G15),"")</f>
+        <v/>
+      </c>
+      <c r="K15" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E15,'Repos to Import'!$A$4:$A$14,0))="",H15=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E15,'Repos to Import'!$A$4:$A$14,0))&amp;H15),"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Presentation-Public-Speaking/</t>
         </is>
       </c>
-      <c r="G15" s="11" t="inlineStr">
+      <c r="M15" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Presentation-Public-Speaking/web/</t>
         </is>
       </c>
-      <c r="H15" s="11" t="inlineStr">
+      <c r="N15" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Presentation-Public-Speaking/facilitator/</t>
         </is>
-      </c>
-      <c r="I15" s="11" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-presentation-public-speaking.html</t>
-        </is>
-      </c>
-      <c r="J15" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E15,'Repos to Import'!$A$4:$A$14,0))="",F15=""),"",SUBSTITUTE(F15,"https://me5231979.github.io/"&amp;$E15&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E15,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K15" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E15,'Repos to Import'!$A$4:$A$14,0))="",G15=""),"",SUBSTITUTE(G15,"https://me5231979.github.io/"&amp;$E15&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E15,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L15" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E15,'Repos to Import'!$A$4:$A$14,0))="",H15=""),"",SUBSTITUTE(H15,"https://me5231979.github.io/"&amp;$E15&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E15,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
       </c>
     </row>
     <row r="16">
@@ -1907,46 +2054,56 @@
           <t>Workflow</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F16" s="27" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G16" s="27" t="inlineStr">
+        <is>
+          <t>/web/</t>
+        </is>
+      </c>
+      <c r="H16" s="27" t="inlineStr">
+        <is>
+          <t>/facilitator/</t>
+        </is>
+      </c>
+      <c r="I16" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E16,'Repos to Import'!$A$4:$A$14,0))="",F16=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E16,'Repos to Import'!$A$4:$A$14,0))&amp;F16),"")</f>
+        <v/>
+      </c>
+      <c r="J16" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E16,'Repos to Import'!$A$4:$A$14,0))="",G16=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E16,'Repos to Import'!$A$4:$A$14,0))&amp;G16),"")</f>
+        <v/>
+      </c>
+      <c r="K16" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E16,'Repos to Import'!$A$4:$A$14,0))="",H16=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E16,'Repos to Import'!$A$4:$A$14,0))&amp;H16),"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Workflow/</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="M16" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Workflow/web/</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="N16" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Workflow/facilitator/</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-workflow-process-redesign.html</t>
-        </is>
-      </c>
-      <c r="J16" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E16,'Repos to Import'!$A$4:$A$14,0))="",F16=""),"",SUBSTITUTE(F16,"https://me5231979.github.io/"&amp;$E16&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E16,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K16" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E16,'Repos to Import'!$A$4:$A$14,0))="",G16=""),"",SUBSTITUTE(G16,"https://me5231979.github.io/"&amp;$E16&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E16,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L16" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E16,'Repos to Import'!$A$4:$A$14,0))="",H16=""),"",SUBSTITUTE(H16,"https://me5231979.github.io/"&amp;$E16&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E16,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
     </row>
     <row r="17">
-      <c r="A17" s="28" t="inlineStr">
+      <c r="A17" s="29" t="inlineStr">
         <is>
           <t>Decisions, Sharper</t>
         </is>
       </c>
-      <c r="B17" s="29" t="inlineStr">
+      <c r="B17" s="30" t="inlineStr">
         <is>
           <t>Manager Voyage</t>
         </is>
@@ -1956,47 +2113,57 @@
           <t>ai leadership</t>
         </is>
       </c>
-      <c r="D17" s="30" t="inlineStr">
+      <c r="D17" s="31" t="inlineStr">
         <is>
           <t>Classroom 45 min · Self-paced ~15 min</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>estesstite</t>
-        </is>
-      </c>
-      <c r="F17" s="11" t="inlineStr">
+          <t>courses</t>
+        </is>
+      </c>
+      <c r="F17" s="32" t="inlineStr">
+        <is>
+          <t>/decisions-class/</t>
+        </is>
+      </c>
+      <c r="G17" s="32" t="inlineStr">
+        <is>
+          <t>/decisions/</t>
+        </is>
+      </c>
+      <c r="H17" s="32" t="inlineStr">
+        <is>
+          <t>/decisions-class/facilitator/</t>
+        </is>
+      </c>
+      <c r="I17" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E17,'Repos to Import'!$A$4:$A$14,0))="",F17=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E17,'Repos to Import'!$A$4:$A$14,0))&amp;F17),"")</f>
+        <v/>
+      </c>
+      <c r="J17" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E17,'Repos to Import'!$A$4:$A$14,0))="",G17=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E17,'Repos to Import'!$A$4:$A$14,0))&amp;G17),"")</f>
+        <v/>
+      </c>
+      <c r="K17" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E17,'Repos to Import'!$A$4:$A$14,0))="",H17=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E17,'Repos to Import'!$A$4:$A$14,0))&amp;H17),"")</f>
+        <v/>
+      </c>
+      <c r="L17" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/decisions-class/</t>
         </is>
       </c>
-      <c r="G17" s="11" t="inlineStr">
+      <c r="M17" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/decisions/</t>
         </is>
       </c>
-      <c r="H17" s="11" t="inlineStr">
+      <c r="N17" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/decisions-class/facilitator/</t>
         </is>
-      </c>
-      <c r="I17" s="11" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-decisions-sharper.html</t>
-        </is>
-      </c>
-      <c r="J17" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E17,'Repos to Import'!$A$4:$A$14,0))="",F17=""),"",SUBSTITUTE(F17,"https://me5231979.github.io/"&amp;$E17&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E17,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K17" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E17,'Repos to Import'!$A$4:$A$14,0))="",G17=""),"",SUBSTITUTE(G17,"https://me5231979.github.io/"&amp;$E17&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E17,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L17" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E17,'Repos to Import'!$A$4:$A$14,0))="",H17=""),"",SUBSTITUTE(H17,"https://me5231979.github.io/"&amp;$E17&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E17,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
       </c>
     </row>
     <row r="18">
@@ -2005,7 +2172,7 @@
           <t>Start Smarter</t>
         </is>
       </c>
-      <c r="B18" s="32" t="inlineStr">
+      <c r="B18" s="34" t="inlineStr">
         <is>
           <t>CHART Program</t>
         </is>
@@ -2025,46 +2192,56 @@
           <t>AI_Classroom</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F18" s="27" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G18" s="27" t="inlineStr">
+        <is>
+          <t>/web/</t>
+        </is>
+      </c>
+      <c r="H18" s="27" t="inlineStr">
+        <is>
+          <t>/facilitator/</t>
+        </is>
+      </c>
+      <c r="I18" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E18,'Repos to Import'!$A$4:$A$14,0))="",F18=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E18,'Repos to Import'!$A$4:$A$14,0))&amp;F18),"")</f>
+        <v/>
+      </c>
+      <c r="J18" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E18,'Repos to Import'!$A$4:$A$14,0))="",G18=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E18,'Repos to Import'!$A$4:$A$14,0))&amp;G18),"")</f>
+        <v/>
+      </c>
+      <c r="K18" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E18,'Repos to Import'!$A$4:$A$14,0))="",H18=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E18,'Repos to Import'!$A$4:$A$14,0))&amp;H18),"")</f>
+        <v/>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/AI_Classroom/</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="M18" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/AI_Classroom/web/</t>
         </is>
       </c>
-      <c r="H18" s="5" t="inlineStr">
+      <c r="N18" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/AI_Classroom/facilitator/</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-start-smarter.html</t>
-        </is>
-      </c>
-      <c r="J18" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E18,'Repos to Import'!$A$4:$A$14,0))="",F18=""),"",SUBSTITUTE(F18,"https://me5231979.github.io/"&amp;$E18&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E18,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K18" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E18,'Repos to Import'!$A$4:$A$14,0))="",G18=""),"",SUBSTITUTE(G18,"https://me5231979.github.io/"&amp;$E18&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E18,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L18" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E18,'Repos to Import'!$A$4:$A$14,0))="",H18=""),"",SUBSTITUTE(H18,"https://me5231979.github.io/"&amp;$E18&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E18,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
     </row>
     <row r="19">
-      <c r="A19" s="28" t="inlineStr">
+      <c r="A19" s="29" t="inlineStr">
         <is>
           <t>Across Your Week</t>
         </is>
       </c>
-      <c r="B19" s="33" t="inlineStr">
+      <c r="B19" s="35" t="inlineStr">
         <is>
           <t>CHART Program</t>
         </is>
@@ -2074,7 +2251,7 @@
           <t>ai</t>
         </is>
       </c>
-      <c r="D19" s="30" t="inlineStr">
+      <c r="D19" s="31" t="inlineStr">
         <is>
           <t>Classroom 90 min · Self-paced ~45 min</t>
         </is>
@@ -2084,37 +2261,47 @@
           <t>Course_Library</t>
         </is>
       </c>
-      <c r="F19" s="11" t="inlineStr">
+      <c r="F19" s="32" t="inlineStr">
+        <is>
+          <t>/courses/AI-Across-Your-Week/</t>
+        </is>
+      </c>
+      <c r="G19" s="32" t="inlineStr">
+        <is>
+          <t>/courses/AI-Across-Your-Week/web/</t>
+        </is>
+      </c>
+      <c r="H19" s="32" t="inlineStr">
+        <is>
+          <t>/courses/AI-Across-Your-Week/facilitator/</t>
+        </is>
+      </c>
+      <c r="I19" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E19,'Repos to Import'!$A$4:$A$14,0))="",F19=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E19,'Repos to Import'!$A$4:$A$14,0))&amp;F19),"")</f>
+        <v/>
+      </c>
+      <c r="J19" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E19,'Repos to Import'!$A$4:$A$14,0))="",G19=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E19,'Repos to Import'!$A$4:$A$14,0))&amp;G19),"")</f>
+        <v/>
+      </c>
+      <c r="K19" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E19,'Repos to Import'!$A$4:$A$14,0))="",H19=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E19,'Repos to Import'!$A$4:$A$14,0))&amp;H19),"")</f>
+        <v/>
+      </c>
+      <c r="L19" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/AI-Across-Your-Week/</t>
         </is>
       </c>
-      <c r="G19" s="11" t="inlineStr">
+      <c r="M19" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/AI-Across-Your-Week/web/</t>
         </is>
       </c>
-      <c r="H19" s="11" t="inlineStr">
+      <c r="N19" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/AI-Across-Your-Week/facilitator/</t>
         </is>
-      </c>
-      <c r="I19" s="11" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-ai-across-your-week.html</t>
-        </is>
-      </c>
-      <c r="J19" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E19,'Repos to Import'!$A$4:$A$14,0))="",F19=""),"",SUBSTITUTE(F19,"https://me5231979.github.io/"&amp;$E19&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E19,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K19" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E19,'Repos to Import'!$A$4:$A$14,0))="",G19=""),"",SUBSTITUTE(G19,"https://me5231979.github.io/"&amp;$E19&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E19,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L19" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E19,'Repos to Import'!$A$4:$A$14,0))="",H19=""),"",SUBSTITUTE(H19,"https://me5231979.github.io/"&amp;$E19&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E19,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
       </c>
     </row>
     <row r="20">
@@ -2123,7 +2310,7 @@
           <t>Admin, Automated</t>
         </is>
       </c>
-      <c r="B20" s="32" t="inlineStr">
+      <c r="B20" s="34" t="inlineStr">
         <is>
           <t>CHART Program</t>
         </is>
@@ -2143,46 +2330,56 @@
           <t>Course_Library</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F20" s="27" t="inlineStr">
+        <is>
+          <t>/courses/Admin-Automated/</t>
+        </is>
+      </c>
+      <c r="G20" s="27" t="inlineStr">
+        <is>
+          <t>/courses/Admin-Automated/web/</t>
+        </is>
+      </c>
+      <c r="H20" s="27" t="inlineStr">
+        <is>
+          <t>/courses/Admin-Automated/facilitator/</t>
+        </is>
+      </c>
+      <c r="I20" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E20,'Repos to Import'!$A$4:$A$14,0))="",F20=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E20,'Repos to Import'!$A$4:$A$14,0))&amp;F20),"")</f>
+        <v/>
+      </c>
+      <c r="J20" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E20,'Repos to Import'!$A$4:$A$14,0))="",G20=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E20,'Repos to Import'!$A$4:$A$14,0))&amp;G20),"")</f>
+        <v/>
+      </c>
+      <c r="K20" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E20,'Repos to Import'!$A$4:$A$14,0))="",H20=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E20,'Repos to Import'!$A$4:$A$14,0))&amp;H20),"")</f>
+        <v/>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Admin-Automated/</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="M20" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Admin-Automated/web/</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="N20" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Admin-Automated/facilitator/</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-admin-automated.html</t>
-        </is>
-      </c>
-      <c r="J20" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E20,'Repos to Import'!$A$4:$A$14,0))="",F20=""),"",SUBSTITUTE(F20,"https://me5231979.github.io/"&amp;$E20&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E20,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K20" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E20,'Repos to Import'!$A$4:$A$14,0))="",G20=""),"",SUBSTITUTE(G20,"https://me5231979.github.io/"&amp;$E20&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E20,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L20" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E20,'Repos to Import'!$A$4:$A$14,0))="",H20=""),"",SUBSTITUTE(H20,"https://me5231979.github.io/"&amp;$E20&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E20,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
     </row>
     <row r="21">
-      <c r="A21" s="28" t="inlineStr">
+      <c r="A21" s="29" t="inlineStr">
         <is>
           <t>Guardrails &amp; Responsible Use</t>
         </is>
       </c>
-      <c r="B21" s="33" t="inlineStr">
+      <c r="B21" s="35" t="inlineStr">
         <is>
           <t>CHART Program</t>
         </is>
@@ -2192,7 +2389,7 @@
           <t>ai</t>
         </is>
       </c>
-      <c r="D21" s="30" t="inlineStr">
+      <c r="D21" s="31" t="inlineStr">
         <is>
           <t>Classroom 90 min · Self-paced ~45 min</t>
         </is>
@@ -2202,37 +2399,47 @@
           <t>Course_Library</t>
         </is>
       </c>
-      <c r="F21" s="11" t="inlineStr">
+      <c r="F21" s="32" t="inlineStr">
+        <is>
+          <t>/courses/AI-Guardrails/</t>
+        </is>
+      </c>
+      <c r="G21" s="32" t="inlineStr">
+        <is>
+          <t>/courses/AI-Guardrails/web/</t>
+        </is>
+      </c>
+      <c r="H21" s="32" t="inlineStr">
+        <is>
+          <t>/courses/AI-Guardrails/facilitator/</t>
+        </is>
+      </c>
+      <c r="I21" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E21,'Repos to Import'!$A$4:$A$14,0))="",F21=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E21,'Repos to Import'!$A$4:$A$14,0))&amp;F21),"")</f>
+        <v/>
+      </c>
+      <c r="J21" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E21,'Repos to Import'!$A$4:$A$14,0))="",G21=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E21,'Repos to Import'!$A$4:$A$14,0))&amp;G21),"")</f>
+        <v/>
+      </c>
+      <c r="K21" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E21,'Repos to Import'!$A$4:$A$14,0))="",H21=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E21,'Repos to Import'!$A$4:$A$14,0))&amp;H21),"")</f>
+        <v/>
+      </c>
+      <c r="L21" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/AI-Guardrails/</t>
         </is>
       </c>
-      <c r="G21" s="11" t="inlineStr">
+      <c r="M21" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/AI-Guardrails/web/</t>
         </is>
       </c>
-      <c r="H21" s="11" t="inlineStr">
+      <c r="N21" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/AI-Guardrails/facilitator/</t>
         </is>
-      </c>
-      <c r="I21" s="11" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-ai-guardrails.html</t>
-        </is>
-      </c>
-      <c r="J21" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E21,'Repos to Import'!$A$4:$A$14,0))="",F21=""),"",SUBSTITUTE(F21,"https://me5231979.github.io/"&amp;$E21&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E21,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K21" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E21,'Repos to Import'!$A$4:$A$14,0))="",G21=""),"",SUBSTITUTE(G21,"https://me5231979.github.io/"&amp;$E21&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E21,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L21" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E21,'Repos to Import'!$A$4:$A$14,0))="",H21=""),"",SUBSTITUTE(H21,"https://me5231979.github.io/"&amp;$E21&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E21,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
       </c>
     </row>
     <row r="22">
@@ -2241,7 +2448,7 @@
           <t>Numbers, Faster</t>
         </is>
       </c>
-      <c r="B22" s="32" t="inlineStr">
+      <c r="B22" s="34" t="inlineStr">
         <is>
           <t>CHART Program</t>
         </is>
@@ -2261,46 +2468,56 @@
           <t>Course_Library</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F22" s="27" t="inlineStr">
+        <is>
+          <t>/courses/Numbers-Faster/</t>
+        </is>
+      </c>
+      <c r="G22" s="27" t="inlineStr">
+        <is>
+          <t>/courses/Numbers-Faster/web/</t>
+        </is>
+      </c>
+      <c r="H22" s="27" t="inlineStr">
+        <is>
+          <t>/courses/Numbers-Faster/facilitator/</t>
+        </is>
+      </c>
+      <c r="I22" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E22,'Repos to Import'!$A$4:$A$14,0))="",F22=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E22,'Repos to Import'!$A$4:$A$14,0))&amp;F22),"")</f>
+        <v/>
+      </c>
+      <c r="J22" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E22,'Repos to Import'!$A$4:$A$14,0))="",G22=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E22,'Repos to Import'!$A$4:$A$14,0))&amp;G22),"")</f>
+        <v/>
+      </c>
+      <c r="K22" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E22,'Repos to Import'!$A$4:$A$14,0))="",H22=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E22,'Repos to Import'!$A$4:$A$14,0))&amp;H22),"")</f>
+        <v/>
+      </c>
+      <c r="L22" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Numbers-Faster/</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="M22" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Numbers-Faster/web/</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="N22" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Numbers-Faster/facilitator/</t>
         </is>
       </c>
-      <c r="I22" s="5" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-numbers-faster.html</t>
-        </is>
-      </c>
-      <c r="J22" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E22,'Repos to Import'!$A$4:$A$14,0))="",F22=""),"",SUBSTITUTE(F22,"https://me5231979.github.io/"&amp;$E22&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E22,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K22" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E22,'Repos to Import'!$A$4:$A$14,0))="",G22=""),"",SUBSTITUTE(G22,"https://me5231979.github.io/"&amp;$E22&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E22,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L22" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E22,'Repos to Import'!$A$4:$A$14,0))="",H22=""),"",SUBSTITUTE(H22,"https://me5231979.github.io/"&amp;$E22&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E22,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
     </row>
     <row r="23">
-      <c r="A23" s="28" t="inlineStr">
+      <c r="A23" s="29" t="inlineStr">
         <is>
           <t>Trust, Then Verify</t>
         </is>
       </c>
-      <c r="B23" s="33" t="inlineStr">
+      <c r="B23" s="35" t="inlineStr">
         <is>
           <t>CHART Program</t>
         </is>
@@ -2310,7 +2527,7 @@
           <t>ai</t>
         </is>
       </c>
-      <c r="D23" s="30" t="inlineStr">
+      <c r="D23" s="31" t="inlineStr">
         <is>
           <t>Classroom 90 min · Self-paced ~45 min</t>
         </is>
@@ -2320,37 +2537,47 @@
           <t>Course_Library</t>
         </is>
       </c>
-      <c r="F23" s="11" t="inlineStr">
+      <c r="F23" s="32" t="inlineStr">
+        <is>
+          <t>/courses/Trust-Then-Verify/</t>
+        </is>
+      </c>
+      <c r="G23" s="32" t="inlineStr">
+        <is>
+          <t>/courses/Trust-Then-Verify/web/</t>
+        </is>
+      </c>
+      <c r="H23" s="32" t="inlineStr">
+        <is>
+          <t>/courses/Trust-Then-Verify/facilitator/</t>
+        </is>
+      </c>
+      <c r="I23" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E23,'Repos to Import'!$A$4:$A$14,0))="",F23=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E23,'Repos to Import'!$A$4:$A$14,0))&amp;F23),"")</f>
+        <v/>
+      </c>
+      <c r="J23" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E23,'Repos to Import'!$A$4:$A$14,0))="",G23=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E23,'Repos to Import'!$A$4:$A$14,0))&amp;G23),"")</f>
+        <v/>
+      </c>
+      <c r="K23" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E23,'Repos to Import'!$A$4:$A$14,0))="",H23=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E23,'Repos to Import'!$A$4:$A$14,0))&amp;H23),"")</f>
+        <v/>
+      </c>
+      <c r="L23" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Trust-Then-Verify/</t>
         </is>
       </c>
-      <c r="G23" s="11" t="inlineStr">
+      <c r="M23" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Trust-Then-Verify/web/</t>
         </is>
       </c>
-      <c r="H23" s="11" t="inlineStr">
+      <c r="N23" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/Course_Library/courses/Trust-Then-Verify/facilitator/</t>
         </is>
-      </c>
-      <c r="I23" s="11" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-trust-then-verify.html</t>
-        </is>
-      </c>
-      <c r="J23" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E23,'Repos to Import'!$A$4:$A$14,0))="",F23=""),"",SUBSTITUTE(F23,"https://me5231979.github.io/"&amp;$E23&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E23,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K23" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E23,'Repos to Import'!$A$4:$A$14,0))="",G23=""),"",SUBSTITUTE(G23,"https://me5231979.github.io/"&amp;$E23&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E23,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L23" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E23,'Repos to Import'!$A$4:$A$14,0))="",H23=""),"",SUBSTITUTE(H23,"https://me5231979.github.io/"&amp;$E23&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E23,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
       </c>
     </row>
     <row r="24">
@@ -2359,7 +2586,7 @@
           <t>Answers, Faster</t>
         </is>
       </c>
-      <c r="B24" s="32" t="inlineStr">
+      <c r="B24" s="34" t="inlineStr">
         <is>
           <t>CHART Program</t>
         </is>
@@ -2376,49 +2603,59 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>estesstite</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
+          <t>courses</t>
+        </is>
+      </c>
+      <c r="F24" s="27" t="inlineStr">
+        <is>
+          <t>/answers-class/</t>
+        </is>
+      </c>
+      <c r="G24" s="27" t="inlineStr">
+        <is>
+          <t>/answers/</t>
+        </is>
+      </c>
+      <c r="H24" s="27" t="inlineStr">
+        <is>
+          <t>/answers-class/facilitator/</t>
+        </is>
+      </c>
+      <c r="I24" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E24,'Repos to Import'!$A$4:$A$14,0))="",F24=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E24,'Repos to Import'!$A$4:$A$14,0))&amp;F24),"")</f>
+        <v/>
+      </c>
+      <c r="J24" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E24,'Repos to Import'!$A$4:$A$14,0))="",G24=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E24,'Repos to Import'!$A$4:$A$14,0))&amp;G24),"")</f>
+        <v/>
+      </c>
+      <c r="K24" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E24,'Repos to Import'!$A$4:$A$14,0))="",H24=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E24,'Repos to Import'!$A$4:$A$14,0))&amp;H24),"")</f>
+        <v/>
+      </c>
+      <c r="L24" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/answers-class/</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="M24" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/answers/</t>
         </is>
       </c>
-      <c r="H24" s="5" t="inlineStr">
+      <c r="N24" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/answers-class/facilitator/</t>
         </is>
       </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-answers-faster.html</t>
-        </is>
-      </c>
-      <c r="J24" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E24,'Repos to Import'!$A$4:$A$14,0))="",F24=""),"",SUBSTITUTE(F24,"https://me5231979.github.io/"&amp;$E24&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E24,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K24" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E24,'Repos to Import'!$A$4:$A$14,0))="",G24=""),"",SUBSTITUTE(G24,"https://me5231979.github.io/"&amp;$E24&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E24,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L24" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E24,'Repos to Import'!$A$4:$A$14,0))="",H24=""),"",SUBSTITUTE(H24,"https://me5231979.github.io/"&amp;$E24&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E24,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
     </row>
     <row r="25">
-      <c r="A25" s="28" t="inlineStr">
+      <c r="A25" s="29" t="inlineStr">
         <is>
           <t>First Drafts, Faster</t>
         </is>
       </c>
-      <c r="B25" s="33" t="inlineStr">
+      <c r="B25" s="35" t="inlineStr">
         <is>
           <t>CHART Program</t>
         </is>
@@ -2428,47 +2665,57 @@
           <t>ai communication</t>
         </is>
       </c>
-      <c r="D25" s="30" t="inlineStr">
+      <c r="D25" s="31" t="inlineStr">
         <is>
           <t>Classroom 45 min · Self-paced ~15 min</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>estesstite</t>
-        </is>
-      </c>
-      <c r="F25" s="11" t="inlineStr">
+          <t>courses</t>
+        </is>
+      </c>
+      <c r="F25" s="32" t="inlineStr">
+        <is>
+          <t>/drafts-class/</t>
+        </is>
+      </c>
+      <c r="G25" s="32" t="inlineStr">
+        <is>
+          <t>/drafts/</t>
+        </is>
+      </c>
+      <c r="H25" s="32" t="inlineStr">
+        <is>
+          <t>/drafts-class/facilitator/</t>
+        </is>
+      </c>
+      <c r="I25" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E25,'Repos to Import'!$A$4:$A$14,0))="",F25=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E25,'Repos to Import'!$A$4:$A$14,0))&amp;F25),"")</f>
+        <v/>
+      </c>
+      <c r="J25" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E25,'Repos to Import'!$A$4:$A$14,0))="",G25=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E25,'Repos to Import'!$A$4:$A$14,0))&amp;G25),"")</f>
+        <v/>
+      </c>
+      <c r="K25" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E25,'Repos to Import'!$A$4:$A$14,0))="",H25=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E25,'Repos to Import'!$A$4:$A$14,0))&amp;H25),"")</f>
+        <v/>
+      </c>
+      <c r="L25" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/drafts-class/</t>
         </is>
       </c>
-      <c r="G25" s="11" t="inlineStr">
+      <c r="M25" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/drafts/</t>
         </is>
       </c>
-      <c r="H25" s="11" t="inlineStr">
+      <c r="N25" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/drafts-class/facilitator/</t>
         </is>
-      </c>
-      <c r="I25" s="11" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-first-drafts-faster.html</t>
-        </is>
-      </c>
-      <c r="J25" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E25,'Repos to Import'!$A$4:$A$14,0))="",F25=""),"",SUBSTITUTE(F25,"https://me5231979.github.io/"&amp;$E25&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E25,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K25" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E25,'Repos to Import'!$A$4:$A$14,0))="",G25=""),"",SUBSTITUTE(G25,"https://me5231979.github.io/"&amp;$E25&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E25,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L25" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E25,'Repos to Import'!$A$4:$A$14,0))="",H25=""),"",SUBSTITUTE(H25,"https://me5231979.github.io/"&amp;$E25&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E25,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
       </c>
     </row>
     <row r="26">
@@ -2477,7 +2724,7 @@
           <t>Ideas, Faster</t>
         </is>
       </c>
-      <c r="B26" s="32" t="inlineStr">
+      <c r="B26" s="34" t="inlineStr">
         <is>
           <t>CHART Program</t>
         </is>
@@ -2494,49 +2741,59 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>estesstite</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
+          <t>courses</t>
+        </is>
+      </c>
+      <c r="F26" s="27" t="inlineStr">
+        <is>
+          <t>/ideas-class/</t>
+        </is>
+      </c>
+      <c r="G26" s="27" t="inlineStr">
+        <is>
+          <t>/ideas/</t>
+        </is>
+      </c>
+      <c r="H26" s="27" t="inlineStr">
+        <is>
+          <t>/ideas-class/facilitator/</t>
+        </is>
+      </c>
+      <c r="I26" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E26,'Repos to Import'!$A$4:$A$14,0))="",F26=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E26,'Repos to Import'!$A$4:$A$14,0))&amp;F26),"")</f>
+        <v/>
+      </c>
+      <c r="J26" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E26,'Repos to Import'!$A$4:$A$14,0))="",G26=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E26,'Repos to Import'!$A$4:$A$14,0))&amp;G26),"")</f>
+        <v/>
+      </c>
+      <c r="K26" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E26,'Repos to Import'!$A$4:$A$14,0))="",H26=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E26,'Repos to Import'!$A$4:$A$14,0))&amp;H26),"")</f>
+        <v/>
+      </c>
+      <c r="L26" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/ideas-class/</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="M26" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/ideas/</t>
         </is>
       </c>
-      <c r="H26" s="5" t="inlineStr">
+      <c r="N26" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/ideas-class/facilitator/</t>
         </is>
       </c>
-      <c r="I26" s="5" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-ideas-faster.html</t>
-        </is>
-      </c>
-      <c r="J26" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E26,'Repos to Import'!$A$4:$A$14,0))="",F26=""),"",SUBSTITUTE(F26,"https://me5231979.github.io/"&amp;$E26&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E26,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K26" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E26,'Repos to Import'!$A$4:$A$14,0))="",G26=""),"",SUBSTITUTE(G26,"https://me5231979.github.io/"&amp;$E26&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E26,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L26" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E26,'Repos to Import'!$A$4:$A$14,0))="",H26=""),"",SUBSTITUTE(H26,"https://me5231979.github.io/"&amp;$E26&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E26,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
     </row>
     <row r="27">
-      <c r="A27" s="28" t="inlineStr">
+      <c r="A27" s="29" t="inlineStr">
         <is>
           <t>Minutes, Faster</t>
         </is>
       </c>
-      <c r="B27" s="33" t="inlineStr">
+      <c r="B27" s="35" t="inlineStr">
         <is>
           <t>CHART Program</t>
         </is>
@@ -2546,47 +2803,57 @@
           <t>ai communication</t>
         </is>
       </c>
-      <c r="D27" s="30" t="inlineStr">
+      <c r="D27" s="31" t="inlineStr">
         <is>
           <t>Classroom 45 min · Self-paced ~15 min</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>estesstite</t>
-        </is>
-      </c>
-      <c r="F27" s="11" t="inlineStr">
+          <t>courses</t>
+        </is>
+      </c>
+      <c r="F27" s="32" t="inlineStr">
+        <is>
+          <t>/minutes-class/</t>
+        </is>
+      </c>
+      <c r="G27" s="32" t="inlineStr">
+        <is>
+          <t>/minutes/</t>
+        </is>
+      </c>
+      <c r="H27" s="32" t="inlineStr">
+        <is>
+          <t>/minutes-class/facilitator/</t>
+        </is>
+      </c>
+      <c r="I27" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E27,'Repos to Import'!$A$4:$A$14,0))="",F27=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E27,'Repos to Import'!$A$4:$A$14,0))&amp;F27),"")</f>
+        <v/>
+      </c>
+      <c r="J27" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E27,'Repos to Import'!$A$4:$A$14,0))="",G27=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E27,'Repos to Import'!$A$4:$A$14,0))&amp;G27),"")</f>
+        <v/>
+      </c>
+      <c r="K27" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E27,'Repos to Import'!$A$4:$A$14,0))="",H27=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E27,'Repos to Import'!$A$4:$A$14,0))&amp;H27),"")</f>
+        <v/>
+      </c>
+      <c r="L27" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/minutes-class/</t>
         </is>
       </c>
-      <c r="G27" s="11" t="inlineStr">
+      <c r="M27" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/minutes/</t>
         </is>
       </c>
-      <c r="H27" s="11" t="inlineStr">
+      <c r="N27" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/minutes-class/facilitator/</t>
         </is>
-      </c>
-      <c r="I27" s="11" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-minutes-faster.html</t>
-        </is>
-      </c>
-      <c r="J27" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E27,'Repos to Import'!$A$4:$A$14,0))="",F27=""),"",SUBSTITUTE(F27,"https://me5231979.github.io/"&amp;$E27&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E27,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K27" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E27,'Repos to Import'!$A$4:$A$14,0))="",G27=""),"",SUBSTITUTE(G27,"https://me5231979.github.io/"&amp;$E27&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E27,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L27" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E27,'Repos to Import'!$A$4:$A$14,0))="",H27=""),"",SUBSTITUTE(H27,"https://me5231979.github.io/"&amp;$E27&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E27,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
       </c>
     </row>
     <row r="28">
@@ -2595,7 +2862,7 @@
           <t>Slides, Faster</t>
         </is>
       </c>
-      <c r="B28" s="32" t="inlineStr">
+      <c r="B28" s="34" t="inlineStr">
         <is>
           <t>CHART Program</t>
         </is>
@@ -2612,49 +2879,59 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>estesstite</t>
-        </is>
-      </c>
-      <c r="F28" s="5" t="inlineStr">
+          <t>courses</t>
+        </is>
+      </c>
+      <c r="F28" s="27" t="inlineStr">
+        <is>
+          <t>/slides-class/</t>
+        </is>
+      </c>
+      <c r="G28" s="27" t="inlineStr">
+        <is>
+          <t>/slides/</t>
+        </is>
+      </c>
+      <c r="H28" s="27" t="inlineStr">
+        <is>
+          <t>/slides-class/facilitator/</t>
+        </is>
+      </c>
+      <c r="I28" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E28,'Repos to Import'!$A$4:$A$14,0))="",F28=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E28,'Repos to Import'!$A$4:$A$14,0))&amp;F28),"")</f>
+        <v/>
+      </c>
+      <c r="J28" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E28,'Repos to Import'!$A$4:$A$14,0))="",G28=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E28,'Repos to Import'!$A$4:$A$14,0))&amp;G28),"")</f>
+        <v/>
+      </c>
+      <c r="K28" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E28,'Repos to Import'!$A$4:$A$14,0))="",H28=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E28,'Repos to Import'!$A$4:$A$14,0))&amp;H28),"")</f>
+        <v/>
+      </c>
+      <c r="L28" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/slides-class/</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="M28" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/slides/</t>
         </is>
       </c>
-      <c r="H28" s="5" t="inlineStr">
+      <c r="N28" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/slides-class/facilitator/</t>
         </is>
       </c>
-      <c r="I28" s="5" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-slides-faster.html</t>
-        </is>
-      </c>
-      <c r="J28" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E28,'Repos to Import'!$A$4:$A$14,0))="",F28=""),"",SUBSTITUTE(F28,"https://me5231979.github.io/"&amp;$E28&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E28,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K28" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E28,'Repos to Import'!$A$4:$A$14,0))="",G28=""),"",SUBSTITUTE(G28,"https://me5231979.github.io/"&amp;$E28&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E28,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L28" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E28,'Repos to Import'!$A$4:$A$14,0))="",H28=""),"",SUBSTITUTE(H28,"https://me5231979.github.io/"&amp;$E28&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E28,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
     </row>
     <row r="29">
-      <c r="A29" s="28" t="inlineStr">
+      <c r="A29" s="29" t="inlineStr">
         <is>
           <t>Working Smarter</t>
         </is>
       </c>
-      <c r="B29" s="33" t="inlineStr">
+      <c r="B29" s="35" t="inlineStr">
         <is>
           <t>CHART Program</t>
         </is>
@@ -2664,47 +2941,57 @@
           <t>ai</t>
         </is>
       </c>
-      <c r="D29" s="30" t="inlineStr">
+      <c r="D29" s="31" t="inlineStr">
         <is>
           <t>Classroom 60&amp;ndash;90 min · Self-paced 60&amp;ndash;90 min</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>estesstite</t>
-        </is>
-      </c>
-      <c r="F29" s="11" t="inlineStr">
+          <t>courses</t>
+        </is>
+      </c>
+      <c r="F29" s="32" t="inlineStr">
+        <is>
+          <t>/classroom/</t>
+        </is>
+      </c>
+      <c r="G29" s="32" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="H29" s="32" t="inlineStr">
+        <is>
+          <t>/classroom/facilitator/</t>
+        </is>
+      </c>
+      <c r="I29" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E29,'Repos to Import'!$A$4:$A$14,0))="",F29=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E29,'Repos to Import'!$A$4:$A$14,0))&amp;F29),"")</f>
+        <v/>
+      </c>
+      <c r="J29" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E29,'Repos to Import'!$A$4:$A$14,0))="",G29=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E29,'Repos to Import'!$A$4:$A$14,0))&amp;G29),"")</f>
+        <v/>
+      </c>
+      <c r="K29" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E29,'Repos to Import'!$A$4:$A$14,0))="",H29=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E29,'Repos to Import'!$A$4:$A$14,0))&amp;H29),"")</f>
+        <v/>
+      </c>
+      <c r="L29" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/classroom/</t>
         </is>
       </c>
-      <c r="G29" s="11" t="inlineStr">
+      <c r="M29" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/</t>
         </is>
       </c>
-      <c r="H29" s="11" t="inlineStr">
+      <c r="N29" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/estesstite/learn/classroom/facilitator/</t>
         </is>
-      </c>
-      <c r="I29" s="11" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-working-smarter.html</t>
-        </is>
-      </c>
-      <c r="J29" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E29,'Repos to Import'!$A$4:$A$14,0))="",F29=""),"",SUBSTITUTE(F29,"https://me5231979.github.io/"&amp;$E29&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E29,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K29" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E29,'Repos to Import'!$A$4:$A$14,0))="",G29=""),"",SUBSTITUTE(G29,"https://me5231979.github.io/"&amp;$E29&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E29,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L29" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E29,'Repos to Import'!$A$4:$A$14,0))="",H29=""),"",SUBSTITUTE(H29,"https://me5231979.github.io/"&amp;$E29&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E29,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
       </c>
     </row>
     <row r="30">
@@ -2713,7 +3000,7 @@
           <t>HCM Essentials</t>
         </is>
       </c>
-      <c r="B30" s="32" t="inlineStr">
+      <c r="B30" s="34" t="inlineStr">
         <is>
           <t>Standalone</t>
         </is>
@@ -2733,46 +3020,56 @@
           <t>HCM_Education</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="F30" s="27" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G30" s="27" t="inlineStr">
+        <is>
+          <t>/web/</t>
+        </is>
+      </c>
+      <c r="H30" s="27" t="inlineStr">
+        <is>
+          <t>/facilitator/</t>
+        </is>
+      </c>
+      <c r="I30" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E30,'Repos to Import'!$A$4:$A$14,0))="",F30=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E30,'Repos to Import'!$A$4:$A$14,0))&amp;F30),"")</f>
+        <v/>
+      </c>
+      <c r="J30" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E30,'Repos to Import'!$A$4:$A$14,0))="",G30=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E30,'Repos to Import'!$A$4:$A$14,0))&amp;G30),"")</f>
+        <v/>
+      </c>
+      <c r="K30" s="28">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E30,'Repos to Import'!$A$4:$A$14,0))="",H30=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E30,'Repos to Import'!$A$4:$A$14,0))&amp;H30),"")</f>
+        <v/>
+      </c>
+      <c r="L30" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/HCM_Education/</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr">
+      <c r="M30" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/HCM_Education/web/</t>
         </is>
       </c>
-      <c r="H30" s="5" t="inlineStr">
+      <c r="N30" s="5" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/HCM_Education/facilitator/</t>
         </is>
       </c>
-      <c r="I30" s="5" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-hcm-essentials.html</t>
-        </is>
-      </c>
-      <c r="J30" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E30,'Repos to Import'!$A$4:$A$14,0))="",F30=""),"",SUBSTITUTE(F30,"https://me5231979.github.io/"&amp;$E30&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E30,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K30" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E30,'Repos to Import'!$A$4:$A$14,0))="",G30=""),"",SUBSTITUTE(G30,"https://me5231979.github.io/"&amp;$E30&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E30,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L30" s="27">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E30,'Repos to Import'!$A$4:$A$14,0))="",H30=""),"",SUBSTITUTE(H30,"https://me5231979.github.io/"&amp;$E30&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E30,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
     </row>
     <row r="31">
-      <c r="A31" s="28" t="inlineStr">
+      <c r="A31" s="29" t="inlineStr">
         <is>
           <t>Building Brave Teams</t>
         </is>
       </c>
-      <c r="B31" s="33" t="inlineStr">
+      <c r="B31" s="35" t="inlineStr">
         <is>
           <t>Standalone</t>
         </is>
@@ -2782,7 +3079,7 @@
           <t>communication leadership</t>
         </is>
       </c>
-      <c r="D31" s="30" t="inlineStr">
+      <c r="D31" s="31" t="inlineStr">
         <is>
           <t>Classroom 120 min · Self-paced ~60 min</t>
         </is>
@@ -2792,157 +3089,139 @@
           <t>TeamUp</t>
         </is>
       </c>
-      <c r="F31" s="11" t="inlineStr">
+      <c r="F31" s="32" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G31" s="32" t="inlineStr">
+        <is>
+          <t>/web/</t>
+        </is>
+      </c>
+      <c r="H31" s="32" t="inlineStr">
+        <is>
+          <t>/facilitator/</t>
+        </is>
+      </c>
+      <c r="I31" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E31,'Repos to Import'!$A$4:$A$14,0))="",F31=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E31,'Repos to Import'!$A$4:$A$14,0))&amp;F31),"")</f>
+        <v/>
+      </c>
+      <c r="J31" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E31,'Repos to Import'!$A$4:$A$14,0))="",G31=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E31,'Repos to Import'!$A$4:$A$14,0))&amp;G31),"")</f>
+        <v/>
+      </c>
+      <c r="K31" s="33">
+        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E31,'Repos to Import'!$A$4:$A$14,0))="",H31=""),"","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E31,'Repos to Import'!$A$4:$A$14,0))&amp;H31),"")</f>
+        <v/>
+      </c>
+      <c r="L31" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/TeamUp/</t>
         </is>
       </c>
-      <c r="G31" s="11" t="inlineStr">
+      <c r="M31" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/TeamUp/web/</t>
         </is>
       </c>
-      <c r="H31" s="11" t="inlineStr">
+      <c r="N31" s="11" t="inlineStr">
         <is>
           <t>https://me5231979.github.io/TeamUp/facilitator/</t>
         </is>
       </c>
-      <c r="I31" s="11" t="inlineStr">
-        <is>
-          <t>https://me5231979.github.io/Course_Library/syllabus-building-brave-teams.html</t>
-        </is>
-      </c>
-      <c r="J31" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E31,'Repos to Import'!$A$4:$A$14,0))="",F31=""),"",SUBSTITUTE(F31,"https://me5231979.github.io/"&amp;$E31&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E31,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="K31" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E31,'Repos to Import'!$A$4:$A$14,0))="",G31=""),"",SUBSTITUTE(G31,"https://me5231979.github.io/"&amp;$E31&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E31,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
-      <c r="L31" s="31">
-        <f>IFERROR(IF(OR(INDEX('Repos to Import'!$E$4:$E$14,MATCH($E31,'Repos to Import'!$A$4:$A$14,0))="",H31=""),"",SUBSTITUTE(H31,"https://me5231979.github.io/"&amp;$E31&amp;"/","https://"&amp;INDEX('Repos to Import'!$E$4:$E$14,MATCH($E31,'Repos to Import'!$A$4:$A$14,0))&amp;"/")),"")</f>
-        <v/>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:L31"/>
+  <autoFilter ref="A3:N31"/>
   <mergeCells count="1">
-    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A2:N2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId84"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2954,17 +3233,822 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="76" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>What sits at which path, repo by repo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Two repos hold many courses: courses (7) and Course_Library (13). Everything else is one course at the root. Add the path to the end of the domain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="36" t="inlineStr">
+        <is>
+          <t>Course</t>
+        </is>
+      </c>
+      <c r="B3" s="36" t="inlineStr">
+        <is>
+          <t>Classroom</t>
+        </is>
+      </c>
+      <c r="C3" s="36" t="inlineStr">
+        <is>
+          <t>Self-paced</t>
+        </is>
+      </c>
+      <c r="D3" s="36" t="inlineStr">
+        <is>
+          <t>Facilitator</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="37" t="inlineStr">
+        <is>
+          <t>Course_Library   (13 courses)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Across Your Week</t>
+        </is>
+      </c>
+      <c r="B5" s="38" t="inlineStr">
+        <is>
+          <t>/courses/AI-Across-Your-Week/</t>
+        </is>
+      </c>
+      <c r="C5" s="38" t="inlineStr">
+        <is>
+          <t>/courses/AI-Across-Your-Week/web/</t>
+        </is>
+      </c>
+      <c r="D5" s="38" t="inlineStr">
+        <is>
+          <t>/courses/AI-Across-Your-Week/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>Admin, Automated</t>
+        </is>
+      </c>
+      <c r="B6" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Admin-Automated/</t>
+        </is>
+      </c>
+      <c r="C6" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Admin-Automated/web/</t>
+        </is>
+      </c>
+      <c r="D6" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Admin-Automated/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Change That Sticks</t>
+        </is>
+      </c>
+      <c r="B7" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Change-Leadership-for-AI/</t>
+        </is>
+      </c>
+      <c r="C7" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Change-Leadership-for-AI/web/</t>
+        </is>
+      </c>
+      <c r="D7" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Change-Leadership-for-AI/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Delegating, Rethought</t>
+        </is>
+      </c>
+      <c r="B8" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Delegating-with-AI/</t>
+        </is>
+      </c>
+      <c r="C8" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Delegating-with-AI/web/</t>
+        </is>
+      </c>
+      <c r="D8" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Delegating-with-AI/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>Feedback, Ready</t>
+        </is>
+      </c>
+      <c r="B9" s="38" t="inlineStr">
+        <is>
+          <t>/ai-coaching-feedback/</t>
+        </is>
+      </c>
+      <c r="C9" s="38" t="inlineStr">
+        <is>
+          <t>/ai-coaching-feedback/web/</t>
+        </is>
+      </c>
+      <c r="D9" s="38" t="inlineStr">
+        <is>
+          <t>/ai-coaching-feedback/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Guardrails &amp; Responsible Use</t>
+        </is>
+      </c>
+      <c r="B10" s="38" t="inlineStr">
+        <is>
+          <t>/courses/AI-Guardrails/</t>
+        </is>
+      </c>
+      <c r="C10" s="38" t="inlineStr">
+        <is>
+          <t>/courses/AI-Guardrails/web/</t>
+        </is>
+      </c>
+      <c r="D10" s="38" t="inlineStr">
+        <is>
+          <t>/courses/AI-Guardrails/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Hiring, Human</t>
+        </is>
+      </c>
+      <c r="B11" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Hiring-with-AI/</t>
+        </is>
+      </c>
+      <c r="C11" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Hiring-with-AI/web/</t>
+        </is>
+      </c>
+      <c r="D11" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Hiring-with-AI/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Leading the Shift</t>
+        </is>
+      </c>
+      <c r="B12" s="38" t="inlineStr">
+        <is>
+          <t>/leading-ai-adoption/</t>
+        </is>
+      </c>
+      <c r="C12" s="38" t="inlineStr">
+        <is>
+          <t>/leading-ai-adoption/web/</t>
+        </is>
+      </c>
+      <c r="D12" s="38" t="inlineStr">
+        <is>
+          <t>/leading-ai-adoption/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>Making It Normal</t>
+        </is>
+      </c>
+      <c r="B13" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Leading-AI-Adoption/</t>
+        </is>
+      </c>
+      <c r="C13" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Leading-AI-Adoption/web/</t>
+        </is>
+      </c>
+      <c r="D13" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Leading-AI-Adoption/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Numbers, Faster</t>
+        </is>
+      </c>
+      <c r="B14" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Numbers-Faster/</t>
+        </is>
+      </c>
+      <c r="C14" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Numbers-Faster/web/</t>
+        </is>
+      </c>
+      <c r="D14" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Numbers-Faster/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>People Data, Safely</t>
+        </is>
+      </c>
+      <c r="B15" s="38" t="inlineStr">
+        <is>
+          <t>/courses/People-Data-with-AI/</t>
+        </is>
+      </c>
+      <c r="C15" s="38" t="inlineStr">
+        <is>
+          <t>/courses/People-Data-with-AI/web/</t>
+        </is>
+      </c>
+      <c r="D15" s="38" t="inlineStr">
+        <is>
+          <t>/courses/People-Data-with-AI/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Talent Calls, Sharper</t>
+        </is>
+      </c>
+      <c r="B16" s="38" t="inlineStr">
+        <is>
+          <t>/ai-talent-decisions/</t>
+        </is>
+      </c>
+      <c r="C16" s="38" t="inlineStr">
+        <is>
+          <t>/ai-talent-decisions/web/</t>
+        </is>
+      </c>
+      <c r="D16" s="38" t="inlineStr">
+        <is>
+          <t>/ai-talent-decisions/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Trust, Then Verify</t>
+        </is>
+      </c>
+      <c r="B17" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Trust-Then-Verify/</t>
+        </is>
+      </c>
+      <c r="C17" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Trust-Then-Verify/web/</t>
+        </is>
+      </c>
+      <c r="D17" s="38" t="inlineStr">
+        <is>
+          <t>/courses/Trust-Then-Verify/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="37" t="inlineStr">
+        <is>
+          <t>courses   (7 courses)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Answers, Faster</t>
+        </is>
+      </c>
+      <c r="B20" s="38" t="inlineStr">
+        <is>
+          <t>/answers-class/</t>
+        </is>
+      </c>
+      <c r="C20" s="38" t="inlineStr">
+        <is>
+          <t>/answers/</t>
+        </is>
+      </c>
+      <c r="D20" s="38" t="inlineStr">
+        <is>
+          <t>/answers-class/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Decisions, Sharper</t>
+        </is>
+      </c>
+      <c r="B21" s="38" t="inlineStr">
+        <is>
+          <t>/decisions-class/</t>
+        </is>
+      </c>
+      <c r="C21" s="38" t="inlineStr">
+        <is>
+          <t>/decisions/</t>
+        </is>
+      </c>
+      <c r="D21" s="38" t="inlineStr">
+        <is>
+          <t>/decisions-class/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>First Drafts, Faster</t>
+        </is>
+      </c>
+      <c r="B22" s="38" t="inlineStr">
+        <is>
+          <t>/drafts-class/</t>
+        </is>
+      </c>
+      <c r="C22" s="38" t="inlineStr">
+        <is>
+          <t>/drafts/</t>
+        </is>
+      </c>
+      <c r="D22" s="38" t="inlineStr">
+        <is>
+          <t>/drafts-class/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>Ideas, Faster</t>
+        </is>
+      </c>
+      <c r="B23" s="38" t="inlineStr">
+        <is>
+          <t>/ideas-class/</t>
+        </is>
+      </c>
+      <c r="C23" s="38" t="inlineStr">
+        <is>
+          <t>/ideas/</t>
+        </is>
+      </c>
+      <c r="D23" s="38" t="inlineStr">
+        <is>
+          <t>/ideas-class/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Minutes, Faster</t>
+        </is>
+      </c>
+      <c r="B24" s="38" t="inlineStr">
+        <is>
+          <t>/minutes-class/</t>
+        </is>
+      </c>
+      <c r="C24" s="38" t="inlineStr">
+        <is>
+          <t>/minutes/</t>
+        </is>
+      </c>
+      <c r="D24" s="38" t="inlineStr">
+        <is>
+          <t>/minutes-class/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Slides, Faster</t>
+        </is>
+      </c>
+      <c r="B25" s="38" t="inlineStr">
+        <is>
+          <t>/slides-class/</t>
+        </is>
+      </c>
+      <c r="C25" s="38" t="inlineStr">
+        <is>
+          <t>/slides/</t>
+        </is>
+      </c>
+      <c r="D25" s="38" t="inlineStr">
+        <is>
+          <t>/slides-class/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>Working Smarter</t>
+        </is>
+      </c>
+      <c r="B26" s="38" t="inlineStr">
+        <is>
+          <t>/classroom/</t>
+        </is>
+      </c>
+      <c r="C26" s="38" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="D26" s="38" t="inlineStr">
+        <is>
+          <t>/classroom/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="37" t="inlineStr">
+        <is>
+          <t>AI_Classroom   (1 course)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="18" t="inlineStr">
+        <is>
+          <t>Start Smarter</t>
+        </is>
+      </c>
+      <c r="B29" s="38" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="C29" s="38" t="inlineStr">
+        <is>
+          <t>/web/</t>
+        </is>
+      </c>
+      <c r="D29" s="38" t="inlineStr">
+        <is>
+          <t>/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="37" t="inlineStr">
+        <is>
+          <t>Coaching-for-Performance   (1 course)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="18" t="inlineStr">
+        <is>
+          <t>Coaching for Performance</t>
+        </is>
+      </c>
+      <c r="B32" s="38" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="C32" s="38" t="inlineStr">
+        <is>
+          <t>/web/</t>
+        </is>
+      </c>
+      <c r="D32" s="38" t="inlineStr">
+        <is>
+          <t>/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="37" t="inlineStr">
+        <is>
+          <t>Difficult_Conversations   (1 course)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="18" t="inlineStr">
+        <is>
+          <t>Navigating Difficult Conversations</t>
+        </is>
+      </c>
+      <c r="B35" s="38" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="C35" s="38" t="inlineStr">
+        <is>
+          <t>/web/</t>
+        </is>
+      </c>
+      <c r="D35" s="38" t="inlineStr">
+        <is>
+          <t>/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="37" t="inlineStr">
+        <is>
+          <t>Emotional-Intelligence   (1 course)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="18" t="inlineStr">
+        <is>
+          <t>Emotional Intelligence &amp; Interpersonal Skills</t>
+        </is>
+      </c>
+      <c r="B38" s="38" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="C38" s="38" t="inlineStr">
+        <is>
+          <t>/web/</t>
+        </is>
+      </c>
+      <c r="D38" s="38" t="inlineStr">
+        <is>
+          <t>/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="37" t="inlineStr">
+        <is>
+          <t>HCM_Education   (1 course)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="18" t="inlineStr">
+        <is>
+          <t>HCM Essentials</t>
+        </is>
+      </c>
+      <c r="B41" s="38" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="C41" s="38" t="inlineStr">
+        <is>
+          <t>/web/</t>
+        </is>
+      </c>
+      <c r="D41" s="38" t="inlineStr">
+        <is>
+          <t>/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="37" t="inlineStr">
+        <is>
+          <t>Presentation-Public-Speaking   (1 course)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="18" t="inlineStr">
+        <is>
+          <t>Presentation &amp; Public Speaking</t>
+        </is>
+      </c>
+      <c r="B44" s="38" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="C44" s="38" t="inlineStr">
+        <is>
+          <t>/web/</t>
+        </is>
+      </c>
+      <c r="D44" s="38" t="inlineStr">
+        <is>
+          <t>/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="37" t="inlineStr">
+        <is>
+          <t>TeamUp   (1 course)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="18" t="inlineStr">
+        <is>
+          <t>Building Brave Teams</t>
+        </is>
+      </c>
+      <c r="B47" s="38" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="C47" s="38" t="inlineStr">
+        <is>
+          <t>/web/</t>
+        </is>
+      </c>
+      <c r="D47" s="38" t="inlineStr">
+        <is>
+          <t>/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="37" t="inlineStr">
+        <is>
+          <t>Workflow   (1 course)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="18" t="inlineStr">
+        <is>
+          <t>Workflow &amp; Process Redesign</t>
+        </is>
+      </c>
+      <c r="B50" s="38" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="C50" s="38" t="inlineStr">
+        <is>
+          <t>/web/</t>
+        </is>
+      </c>
+      <c r="D50" s="38" t="inlineStr">
+        <is>
+          <t>/facilitator/</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="21" t="inlineStr">
+        <is>
+          <t>Also on every course built in-house:</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="39" t="inlineStr">
+        <is>
+          <t>/facilitator/guide.html</t>
+        </is>
+      </c>
+      <c r="B53" s="40" t="inlineStr">
+        <is>
+          <t>printable facilitator guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="39" t="inlineStr">
+        <is>
+          <t>/cheatsheet.html</t>
+        </is>
+      </c>
+      <c r="B54" s="40" t="inlineStr">
+        <is>
+          <t>learner cheat sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="39" t="inlineStr">
+        <is>
+          <t>/worksheet.html</t>
+        </is>
+      </c>
+      <c r="B55" s="40" t="inlineStr">
+        <is>
+          <t>learner worksheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="23" t="inlineStr">
+        <is>
+          <t>The CHART courses in the courses repo keep their own structure and do not have these extra pages.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A46:D46"/>
+    <mergeCell ref="A49:D49"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="82" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
           <t>Importing and running these sites</t>
         </is>
       </c>
@@ -2972,10 +4056,10 @@
     <row r="3">
       <c r="A3" s="21" t="inlineStr"/>
       <c r="B3" s="21" t="inlineStr"/>
-      <c r="C3" s="34" t="inlineStr"/>
+      <c r="C3" s="41" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="35" t="inlineStr">
+      <c r="A4" s="37" t="inlineStr">
         <is>
           <t>ONE-COMMAND IMPORT</t>
         </is>
@@ -2992,9 +4076,9 @@
           <t>Make a token</t>
         </is>
       </c>
-      <c r="C5" s="34" t="inlineStr">
-        <is>
-          <t>Vercel &gt; Account Settings &gt; Tokens. Scope it to the FLH team.</t>
+      <c r="C5" s="41" t="inlineStr">
+        <is>
+          <t>Vercel &gt; Account Settings &gt; Tokens, scoped to the FLH team.</t>
         </is>
       </c>
     </row>
@@ -3006,42 +4090,42 @@
       </c>
       <c r="B6" s="21" t="inlineStr">
         <is>
-          <t>Run the script</t>
-        </is>
-      </c>
-      <c r="C6" s="34" t="inlineStr">
-        <is>
-          <t>export VERCEL_TOKEN=...   then   python3 tools/vercel-import.py</t>
+          <t>Run it</t>
+        </is>
+      </c>
+      <c r="C6" s="41" t="inlineStr">
+        <is>
+          <t>export VERCEL_TOKEN=...    then    python3 tools/vercel-import.py</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="21" t="inlineStr"/>
       <c r="B7" s="21" t="inlineStr"/>
-      <c r="C7" s="34" t="inlineStr">
-        <is>
-          <t>Lives in Course_Library/tools/. Safe to re-run: existing projects are skipped.</t>
+      <c r="C7" s="41" t="inlineStr">
+        <is>
+          <t>In Course_Library/tools/. Safe to re-run; existing projects are skipped.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="21" t="inlineStr"/>
       <c r="B8" s="21" t="inlineStr"/>
-      <c r="C8" s="34" t="inlineStr">
-        <is>
-          <t>Add --dry-run first to see the plan without touching anything.</t>
+      <c r="C8" s="41" t="inlineStr">
+        <is>
+          <t>Add --dry-run first to see the plan without creating anything.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="21" t="inlineStr"/>
       <c r="B9" s="21" t="inlineStr"/>
-      <c r="C9" s="34" t="inlineStr"/>
+      <c r="C9" s="41" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="35" t="inlineStr">
-        <is>
-          <t>OR IMPORT BY HAND</t>
+      <c r="A10" s="37" t="inlineStr">
+        <is>
+          <t>OR BY HAND, PER REPO</t>
         </is>
       </c>
     </row>
@@ -3056,9 +4140,9 @@
           <t>Add New &gt; Project</t>
         </is>
       </c>
-      <c r="C11" s="34" t="inlineStr">
-        <is>
-          <t>Pick the repo from the list on the Repos tab.</t>
+      <c r="C11" s="41" t="inlineStr">
+        <is>
+          <t>Pick the repo from the Repos tab.</t>
         </is>
       </c>
     </row>
@@ -3073,7 +4157,7 @@
           <t>Framework Preset</t>
         </is>
       </c>
-      <c r="C12" s="34" t="inlineStr">
+      <c r="C12" s="41" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
@@ -3090,9 +4174,9 @@
           <t>Root Directory</t>
         </is>
       </c>
-      <c r="C13" s="34" t="inlineStr">
-        <is>
-          <t>LEAVE EMPTY. This is what serves all three editions from one project.</t>
+      <c r="C13" s="41" t="inlineStr">
+        <is>
+          <t>LEAVE EMPTY. This is what serves every edition from one project.</t>
         </is>
       </c>
     </row>
@@ -3104,12 +4188,12 @@
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>Build &amp; Output</t>
-        </is>
-      </c>
-      <c r="C14" s="34" t="inlineStr">
-        <is>
-          <t>No build command, no output directory. The files are pre-generated.</t>
+          <t>Build and Output</t>
+        </is>
+      </c>
+      <c r="C14" s="41" t="inlineStr">
+        <is>
+          <t>No build command, no output directory. Files are pre-generated.</t>
         </is>
       </c>
     </row>
@@ -3124,19 +4208,19 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C15" s="34" t="inlineStr">
-        <is>
-          <t>Then copy the assigned domain into the yellow column on the Repos tab.</t>
+      <c r="C15" s="41" t="inlineStr">
+        <is>
+          <t>Then paste the domain into the yellow column on the Repos tab.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="21" t="inlineStr"/>
       <c r="B16" s="21" t="inlineStr"/>
-      <c r="C16" s="34" t="inlineStr"/>
+      <c r="C16" s="41" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="35" t="inlineStr">
+      <c r="A17" s="37" t="inlineStr">
         <is>
           <t>CHECK ON EVERY PROJECT</t>
         </is>
@@ -3153,7 +4237,7 @@
           <t>Production Branch</t>
         </is>
       </c>
-      <c r="C18" s="34" t="inlineStr">
+      <c r="C18" s="41" t="inlineStr">
         <is>
           <t>Settings &gt; Git. Must be main.</t>
         </is>
@@ -3170,18 +4254,18 @@
           <t>Deployment Protection</t>
         </is>
       </c>
-      <c r="C19" s="34" t="inlineStr">
-        <is>
-          <t>Settings &gt; Deployment Protection &gt; Vercel Authentication =</t>
+      <c r="C19" s="41" t="inlineStr">
+        <is>
+          <t>Vercel Authentication = Only Preview Deployments.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="21" t="inlineStr"/>
       <c r="B20" s="21" t="inlineStr"/>
-      <c r="C20" s="34" t="inlineStr">
-        <is>
-          <t>'Only Preview Deployments'. Otherwise learners scanning a QR code hit a login wall.</t>
+      <c r="C20" s="41" t="inlineStr">
+        <is>
+          <t>Otherwise learners scanning a QR code hit a sign-in wall.</t>
         </is>
       </c>
     </row>
@@ -3193,10 +4277,10 @@
       </c>
       <c r="B21" s="21" t="inlineStr">
         <is>
-          <t>Open it in a private window</t>
-        </is>
-      </c>
-      <c r="C21" s="34" t="inlineStr">
+          <t>Open in a private window</t>
+        </is>
+      </c>
+      <c r="C21" s="41" t="inlineStr">
         <is>
           <t>The real test. If it asks you to sign in, fix (b).</t>
         </is>
@@ -3205,184 +4289,86 @@
     <row r="22">
       <c r="A22" s="21" t="inlineStr"/>
       <c r="B22" s="21" t="inlineStr"/>
-      <c r="C22" s="34" t="inlineStr"/>
+      <c r="C22" s="41" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="35" t="inlineStr">
-        <is>
-          <t>PAGE PATHS ON EVERY COURSE</t>
+      <c r="A23" s="37" t="inlineStr">
+        <is>
+          <t>WHAT MOVED, AND WHAT IS LEFT</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="21" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="A24" s="21" t="inlineStr"/>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>Classroom edition</t>
-        </is>
-      </c>
-      <c r="C24" s="34" t="inlineStr">
-        <is>
-          <t>Projected in the room. Opens on the welcome QR slide.</t>
+          <t>Courses moved</t>
+        </is>
+      </c>
+      <c r="C24" s="41" t="inlineStr">
+        <is>
+          <t>The 7 CHART courses now live in me5231979/courses, one level higher: /learn/drafts-class/ became /drafts-class/.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="21" t="inlineStr">
-        <is>
-          <t>/web/</t>
-        </is>
-      </c>
+      <c r="A25" s="21" t="inlineStr"/>
       <c r="B25" s="21" t="inlineStr">
         <is>
-          <t>Self-paced edition</t>
-        </is>
-      </c>
-      <c r="C25" s="34" t="inlineStr">
-        <is>
-          <t>Same course minus the group prompts.</t>
+          <t>estesstite</t>
+        </is>
+      </c>
+      <c r="C25" s="41" t="inlineStr">
+        <is>
+          <t>Left untouched and still live, so nothing breaks today. Retire it once the catalog links point at the new domain.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="21" t="inlineStr">
-        <is>
-          <t>/facilitator/</t>
-        </is>
-      </c>
+      <c r="A26" s="21" t="inlineStr"/>
       <c r="B26" s="21" t="inlineStr">
         <is>
-          <t>Facilitator edition</t>
-        </is>
-      </c>
-      <c r="C26" s="34" t="inlineStr">
-        <is>
-          <t>Script rail on every slide, prep page first.</t>
+          <t>URL sweep</t>
+        </is>
+      </c>
+      <c r="C26" s="41" t="inlineStr">
+        <is>
+          <t>Facilitator QR codes and every catalog link still point at github.io. One pass fixes them all once domains are settled.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="21" t="inlineStr">
-        <is>
-          <t>/facilitator/guide.html</t>
-        </is>
-      </c>
+      <c r="A27" s="21" t="inlineStr"/>
       <c r="B27" s="21" t="inlineStr">
         <is>
-          <t>Printable guide</t>
-        </is>
-      </c>
-      <c r="C27" s="34" t="inlineStr">
-        <is>
-          <t>Slide image beside the notes, built for paper.</t>
+          <t>Custom domain</t>
+        </is>
+      </c>
+      <c r="C27" s="41" t="inlineStr">
+        <is>
+          <t>Vercel's free names get random suffixes because good ones are taken globally. Your own domain is the permanent fix and makes printed QR codes safe forever.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="21" t="inlineStr">
-        <is>
-          <t>/cheatsheet.html</t>
-        </is>
-      </c>
+      <c r="A28" s="21" t="inlineStr"/>
       <c r="B28" s="21" t="inlineStr">
         <is>
-          <t>Cheat sheet</t>
-        </is>
-      </c>
-      <c r="C28" s="34" t="inlineStr">
-        <is>
-          <t>Learner take-home.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="21" t="inlineStr">
-        <is>
-          <t>/worksheet.html</t>
-        </is>
-      </c>
-      <c r="B29" s="21" t="inlineStr">
-        <is>
-          <t>Worksheet</t>
-        </is>
-      </c>
-      <c r="C29" s="34" t="inlineStr">
-        <is>
-          <t>Learner take-home.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="21" t="inlineStr"/>
-      <c r="B30" s="21" t="inlineStr"/>
-      <c r="C30" s="34" t="inlineStr">
-        <is>
-          <t>The Visit button only opens '/'. Type the rest onto the end of the domain.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="21" t="inlineStr"/>
-      <c r="B31" s="21" t="inlineStr"/>
-      <c r="C31" s="34" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="35" t="inlineStr">
-        <is>
-          <t>STILL TO DO AFTER THE IMPORTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="21" t="inlineStr"/>
-      <c r="B33" s="21" t="inlineStr">
-        <is>
-          <t>URL sweep</t>
-        </is>
-      </c>
-      <c r="C33" s="34" t="inlineStr">
-        <is>
-          <t>Facilitator QR codes and library links still point at github.io. One pass fixes them all once domains are settled.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="21" t="inlineStr"/>
-      <c r="B34" s="21" t="inlineStr">
-        <is>
-          <t>Custom domain</t>
-        </is>
-      </c>
-      <c r="C34" s="34" t="inlineStr">
-        <is>
-          <t>Vercel's free names get random suffixes because the good ones are taken globally. Your own domain is the permanent fix, and it makes printed QR codes safe forever.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="21" t="inlineStr"/>
-      <c r="B35" s="21" t="inlineStr">
-        <is>
-          <t>Make repos private</t>
-        </is>
-      </c>
-      <c r="C35" s="34" t="inlineStr">
-        <is>
-          <t>Safe once Vercel serves the sites. GitHub Pages cannot do private; Vercel can.</t>
+          <t>Private repos</t>
+        </is>
+      </c>
+      <c r="C28" s="41" t="inlineStr">
+        <is>
+          <t>Safe once Vercel serves the sites. GitHub Pages cannot serve private repos; Vercel can.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="4">
     <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A17:C17"/>
     <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A4:C4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Workbook: add the 20 repos to create for one-course-per-repo
Lists every course that still shares a repo, its proposed repo name, and
where it migrates from. Eight courses already stand alone. The 13 coming out
of Course_Library are self-contained and lift cleanly; the 7 CHART courses
need their shared assets copied in and the -class layout normalised.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CHUxqeQb2UgQw5JmmaoKqy
</commit_message>
<xml_diff>
--- a/docs/Vanderbilt-Learning-Series-URLs.xlsx
+++ b/docs/Vanderbilt-Learning-Series-URLs.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Repos to Import" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Course URLs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Paths by Repo" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Setup Checklist" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="New Repos to Create" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Course URLs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Paths by Repo" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Setup Checklist" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Course URLs'!$A$3:$N$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Course URLs'!$A$3:$N$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -105,6 +106,11 @@
       <color rgb="00333333"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Courier New"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -155,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -255,6 +261,15 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -622,7 +637,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
@@ -1095,8 +1110,694 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Create these 20 repos, one per course</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Create each as EMPTY under github.com/me5231979 (no README, no .gitignore, no license). Tell me which ones exist and I migrate the course in, keeping every edition, then it becomes its own Vercel project. Eight courses already have their own repo and are not listed here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Repo name to create</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Course</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Program</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Migrating from</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Created? (tick)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="42" t="inlineStr">
+        <is>
+          <t>across-your-week</t>
+        </is>
+      </c>
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>Across Your Week</t>
+        </is>
+      </c>
+      <c r="D4" s="34" t="inlineStr">
+        <is>
+          <t>CHART Program</t>
+        </is>
+      </c>
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t>Course_Library/courses/AI-Across-Your-Week/</t>
+        </is>
+      </c>
+      <c r="F4" s="43" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="44" t="inlineStr">
+        <is>
+          <t>admin-automated</t>
+        </is>
+      </c>
+      <c r="C5" s="29" t="inlineStr">
+        <is>
+          <t>Admin, Automated</t>
+        </is>
+      </c>
+      <c r="D5" s="35" t="inlineStr">
+        <is>
+          <t>CHART Program</t>
+        </is>
+      </c>
+      <c r="E5" s="32" t="inlineStr">
+        <is>
+          <t>Course_Library/courses/Admin-Automated/</t>
+        </is>
+      </c>
+      <c r="F5" s="43" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="42" t="inlineStr">
+        <is>
+          <t>change-that-sticks</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>Change That Sticks</t>
+        </is>
+      </c>
+      <c r="D6" s="25" t="inlineStr">
+        <is>
+          <t>Manager Voyage</t>
+        </is>
+      </c>
+      <c r="E6" s="27" t="inlineStr">
+        <is>
+          <t>Course_Library/courses/Change-Leadership-for-AI/</t>
+        </is>
+      </c>
+      <c r="F6" s="43" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="44" t="inlineStr">
+        <is>
+          <t>delegating-rethought</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="inlineStr">
+        <is>
+          <t>Delegating, Rethought</t>
+        </is>
+      </c>
+      <c r="D7" s="30" t="inlineStr">
+        <is>
+          <t>Manager Voyage</t>
+        </is>
+      </c>
+      <c r="E7" s="32" t="inlineStr">
+        <is>
+          <t>Course_Library/courses/Delegating-with-AI/</t>
+        </is>
+      </c>
+      <c r="F7" s="43" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="42" t="inlineStr">
+        <is>
+          <t>feedback-ready</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>Feedback, Ready</t>
+        </is>
+      </c>
+      <c r="D8" s="25" t="inlineStr">
+        <is>
+          <t>Manager Voyage</t>
+        </is>
+      </c>
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>Course_Library/ai-coaching-feedback/</t>
+        </is>
+      </c>
+      <c r="F8" s="43" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="44" t="inlineStr">
+        <is>
+          <t>guardrails-responsible-use</t>
+        </is>
+      </c>
+      <c r="C9" s="29" t="inlineStr">
+        <is>
+          <t>Guardrails &amp; Responsible Use</t>
+        </is>
+      </c>
+      <c r="D9" s="35" t="inlineStr">
+        <is>
+          <t>CHART Program</t>
+        </is>
+      </c>
+      <c r="E9" s="32" t="inlineStr">
+        <is>
+          <t>Course_Library/courses/AI-Guardrails/</t>
+        </is>
+      </c>
+      <c r="F9" s="43" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="42" t="inlineStr">
+        <is>
+          <t>hiring-human</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>Hiring, Human</t>
+        </is>
+      </c>
+      <c r="D10" s="25" t="inlineStr">
+        <is>
+          <t>Manager Voyage</t>
+        </is>
+      </c>
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>Course_Library/courses/Hiring-with-AI/</t>
+        </is>
+      </c>
+      <c r="F10" s="43" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="44" t="inlineStr">
+        <is>
+          <t>leading-the-shift</t>
+        </is>
+      </c>
+      <c r="C11" s="29" t="inlineStr">
+        <is>
+          <t>Leading the Shift</t>
+        </is>
+      </c>
+      <c r="D11" s="30" t="inlineStr">
+        <is>
+          <t>Manager Voyage</t>
+        </is>
+      </c>
+      <c r="E11" s="32" t="inlineStr">
+        <is>
+          <t>Course_Library/leading-ai-adoption/</t>
+        </is>
+      </c>
+      <c r="F11" s="43" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="42" t="inlineStr">
+        <is>
+          <t>making-it-normal</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="inlineStr">
+        <is>
+          <t>Making It Normal</t>
+        </is>
+      </c>
+      <c r="D12" s="25" t="inlineStr">
+        <is>
+          <t>Manager Voyage</t>
+        </is>
+      </c>
+      <c r="E12" s="27" t="inlineStr">
+        <is>
+          <t>Course_Library/courses/Leading-AI-Adoption/</t>
+        </is>
+      </c>
+      <c r="F12" s="43" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="44" t="inlineStr">
+        <is>
+          <t>numbers-faster</t>
+        </is>
+      </c>
+      <c r="C13" s="29" t="inlineStr">
+        <is>
+          <t>Numbers, Faster</t>
+        </is>
+      </c>
+      <c r="D13" s="35" t="inlineStr">
+        <is>
+          <t>CHART Program</t>
+        </is>
+      </c>
+      <c r="E13" s="32" t="inlineStr">
+        <is>
+          <t>Course_Library/courses/Numbers-Faster/</t>
+        </is>
+      </c>
+      <c r="F13" s="43" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="42" t="inlineStr">
+        <is>
+          <t>people-data-safely</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="inlineStr">
+        <is>
+          <t>People Data, Safely</t>
+        </is>
+      </c>
+      <c r="D14" s="25" t="inlineStr">
+        <is>
+          <t>Manager Voyage</t>
+        </is>
+      </c>
+      <c r="E14" s="27" t="inlineStr">
+        <is>
+          <t>Course_Library/courses/People-Data-with-AI/</t>
+        </is>
+      </c>
+      <c r="F14" s="43" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="44" t="inlineStr">
+        <is>
+          <t>talent-calls-sharper</t>
+        </is>
+      </c>
+      <c r="C15" s="29" t="inlineStr">
+        <is>
+          <t>Talent Calls, Sharper</t>
+        </is>
+      </c>
+      <c r="D15" s="30" t="inlineStr">
+        <is>
+          <t>Manager Voyage</t>
+        </is>
+      </c>
+      <c r="E15" s="32" t="inlineStr">
+        <is>
+          <t>Course_Library/ai-talent-decisions/</t>
+        </is>
+      </c>
+      <c r="F15" s="43" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="42" t="inlineStr">
+        <is>
+          <t>trust-then-verify</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="inlineStr">
+        <is>
+          <t>Trust, Then Verify</t>
+        </is>
+      </c>
+      <c r="D16" s="34" t="inlineStr">
+        <is>
+          <t>CHART Program</t>
+        </is>
+      </c>
+      <c r="E16" s="27" t="inlineStr">
+        <is>
+          <t>Course_Library/courses/Trust-Then-Verify/</t>
+        </is>
+      </c>
+      <c r="F16" s="43" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="44" t="inlineStr">
+        <is>
+          <t>answers-faster</t>
+        </is>
+      </c>
+      <c r="C17" s="29" t="inlineStr">
+        <is>
+          <t>Answers, Faster</t>
+        </is>
+      </c>
+      <c r="D17" s="35" t="inlineStr">
+        <is>
+          <t>CHART Program</t>
+        </is>
+      </c>
+      <c r="E17" s="32" t="inlineStr">
+        <is>
+          <t>courses/answers-class/</t>
+        </is>
+      </c>
+      <c r="F17" s="43" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="42" t="inlineStr">
+        <is>
+          <t>decisions-sharper</t>
+        </is>
+      </c>
+      <c r="C18" s="24" t="inlineStr">
+        <is>
+          <t>Decisions, Sharper</t>
+        </is>
+      </c>
+      <c r="D18" s="25" t="inlineStr">
+        <is>
+          <t>Manager Voyage</t>
+        </is>
+      </c>
+      <c r="E18" s="27" t="inlineStr">
+        <is>
+          <t>courses/decisions-class/</t>
+        </is>
+      </c>
+      <c r="F18" s="43" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="44" t="inlineStr">
+        <is>
+          <t>first-drafts-faster</t>
+        </is>
+      </c>
+      <c r="C19" s="29" t="inlineStr">
+        <is>
+          <t>First Drafts, Faster</t>
+        </is>
+      </c>
+      <c r="D19" s="35" t="inlineStr">
+        <is>
+          <t>CHART Program</t>
+        </is>
+      </c>
+      <c r="E19" s="32" t="inlineStr">
+        <is>
+          <t>courses/drafts-class/</t>
+        </is>
+      </c>
+      <c r="F19" s="43" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="42" t="inlineStr">
+        <is>
+          <t>ideas-faster</t>
+        </is>
+      </c>
+      <c r="C20" s="24" t="inlineStr">
+        <is>
+          <t>Ideas, Faster</t>
+        </is>
+      </c>
+      <c r="D20" s="34" t="inlineStr">
+        <is>
+          <t>CHART Program</t>
+        </is>
+      </c>
+      <c r="E20" s="27" t="inlineStr">
+        <is>
+          <t>courses/ideas-class/</t>
+        </is>
+      </c>
+      <c r="F20" s="43" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="44" t="inlineStr">
+        <is>
+          <t>minutes-faster</t>
+        </is>
+      </c>
+      <c r="C21" s="29" t="inlineStr">
+        <is>
+          <t>Minutes, Faster</t>
+        </is>
+      </c>
+      <c r="D21" s="35" t="inlineStr">
+        <is>
+          <t>CHART Program</t>
+        </is>
+      </c>
+      <c r="E21" s="32" t="inlineStr">
+        <is>
+          <t>courses/minutes-class/</t>
+        </is>
+      </c>
+      <c r="F21" s="43" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="42" t="inlineStr">
+        <is>
+          <t>slides-faster</t>
+        </is>
+      </c>
+      <c r="C22" s="24" t="inlineStr">
+        <is>
+          <t>Slides, Faster</t>
+        </is>
+      </c>
+      <c r="D22" s="34" t="inlineStr">
+        <is>
+          <t>CHART Program</t>
+        </is>
+      </c>
+      <c r="E22" s="27" t="inlineStr">
+        <is>
+          <t>courses/slides-class/</t>
+        </is>
+      </c>
+      <c r="F22" s="43" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="44" t="inlineStr">
+        <is>
+          <t>working-smarter</t>
+        </is>
+      </c>
+      <c r="C23" s="29" t="inlineStr">
+        <is>
+          <t>Working Smarter</t>
+        </is>
+      </c>
+      <c r="D23" s="35" t="inlineStr">
+        <is>
+          <t>CHART Program</t>
+        </is>
+      </c>
+      <c r="E23" s="32" t="inlineStr">
+        <is>
+          <t>courses/classroom/</t>
+        </is>
+      </c>
+      <c r="F23" s="43" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="37" t="inlineStr">
+        <is>
+          <t>AFTER MIGRATION, EVERY COURSE LOOKS THE SAME</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="39" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="C26" s="40" t="inlineStr">
+        <is>
+          <t>classroom edition</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="39" t="inlineStr">
+        <is>
+          <t>/web/</t>
+        </is>
+      </c>
+      <c r="C27" s="40" t="inlineStr">
+        <is>
+          <t>self-paced edition</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="39" t="inlineStr">
+        <is>
+          <t>/facilitator/</t>
+        </is>
+      </c>
+      <c r="C28" s="40" t="inlineStr">
+        <is>
+          <t>facilitator edition</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="39" t="inlineStr">
+        <is>
+          <t>/facilitator/guide.html</t>
+        </is>
+      </c>
+      <c r="C29" s="40" t="inlineStr">
+        <is>
+          <t>printable guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="21" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="26" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>The 13 courses coming out of Course_Library are already self-contained: a straight lift, nothing to rewrite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="26" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>The 7 CHART courses share one assets folder and use a -class suffix. Each gets its own copy of the 3 shared files and moves to the layout above, so all 29 courses match.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="26" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Course_Library stays as the catalog only. The courses repo can be retired once all 7 are out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="26" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Repo names are lowercase with hyphens. Rename any of them before you create them and tell me what you used.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A25:F25"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N31"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -3227,14 +3928,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D57"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
@@ -4032,14 +4733,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>

</xml_diff>